<commit_message>
tracking puzzles sheet updates
</commit_message>
<xml_diff>
--- a/docs/Programming Puzzles.xlsx
+++ b/docs/Programming Puzzles.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\ProjectDSA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E64630B-89AE-4A68-8F76-2CD6965B9144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD9A901F-6090-4E21-BF3F-C185C0E7C9CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1228" uniqueCount="423">
   <si>
     <t>PLATFORM</t>
   </si>
@@ -1154,9 +1154,6 @@
     <t>Neetcode 150, Algomonster</t>
   </si>
   <si>
-    <t>In Rating 1 - 5: 1 being very hard, 5 being very easy.</t>
-  </si>
-  <si>
     <t>Dynamic Programming, Backtracking</t>
   </si>
   <si>
@@ -1302,6 +1299,15 @@
   </si>
   <si>
     <t>Hashmaps</t>
+  </si>
+  <si>
+    <t>Anagrams</t>
+  </si>
+  <si>
+    <t>Most Frequent Character</t>
+  </si>
+  <si>
+    <t>In Rating 1 - 5: 1 being very easy, 5 being very hard.</t>
   </si>
 </sst>
 </file>
@@ -1386,7 +1392,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1417,6 +1423,11 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="3" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1756,14 +1767,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E29EE35E-42CE-4BB8-BA9B-83E0DF36D658}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="65.1796875" customWidth="1"/>
+    <col min="1" max="1" width="65.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>371</v>
+        <v>422</v>
       </c>
     </row>
   </sheetData>
@@ -1774,7 +1785,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{673553DD-7322-43E4-B8E6-8596552AA633}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1783,21 +1794,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{758F6333-ADD2-4F62-82FC-3789A0207F8D}">
   <dimension ref="A1:J162"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.453125" customWidth="1"/>
-    <col min="2" max="2" width="11.81640625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="52.26953125" customWidth="1"/>
-    <col min="4" max="4" width="36.453125" customWidth="1"/>
-    <col min="5" max="5" width="13.54296875" customWidth="1"/>
-    <col min="6" max="6" width="13.54296875" style="4" customWidth="1"/>
-    <col min="7" max="7" width="34.54296875" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" style="4" customWidth="1"/>
+    <col min="3" max="3" width="52.28515625" customWidth="1"/>
+    <col min="4" max="4" width="36.42578125" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="34.5703125" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="15.26953125" customWidth="1"/>
-    <col min="10" max="10" width="92.7265625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="15.28515625" customWidth="1"/>
+    <col min="10" max="10" width="92.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1829,7 +1840,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1855,7 +1866,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1866,7 +1877,7 @@
         <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E3" t="s">
         <v>6</v>
@@ -1881,7 +1892,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>5</v>
       </c>
@@ -1892,13 +1903,13 @@
         <v>14</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>6</v>
       </c>
       <c r="F4" s="8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>7</v>
@@ -1907,11 +1918,11 @@
         <v>369</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="J4" s="9"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -1922,7 +1933,7 @@
         <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E5" t="s">
         <v>17</v>
@@ -1937,7 +1948,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1966,7 +1977,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1992,7 +2003,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -2021,7 +2032,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -2050,7 +2061,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -2079,7 +2090,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -2108,7 +2119,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -2137,7 +2148,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>5</v>
       </c>
@@ -2166,10 +2177,10 @@
         <v>42</v>
       </c>
       <c r="J13" s="12" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -2195,7 +2206,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -2224,7 +2235,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -2250,7 +2261,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>5</v>
       </c>
@@ -2279,7 +2290,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>5</v>
       </c>
@@ -2308,7 +2319,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>5</v>
       </c>
@@ -2337,7 +2348,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>5</v>
       </c>
@@ -2366,7 +2377,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>5</v>
       </c>
@@ -2395,7 +2406,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>5</v>
       </c>
@@ -2412,7 +2423,7 @@
         <v>6</v>
       </c>
       <c r="F22" s="8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G22" s="7" t="s">
         <v>7</v>
@@ -2427,7 +2438,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -2456,7 +2467,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>5</v>
       </c>
@@ -2485,7 +2496,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>5</v>
       </c>
@@ -2514,7 +2525,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>5</v>
       </c>
@@ -2540,7 +2551,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>5</v>
       </c>
@@ -2569,7 +2580,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>5</v>
       </c>
@@ -2598,7 +2609,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>5</v>
       </c>
@@ -2627,7 +2638,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>5</v>
       </c>
@@ -2635,7 +2646,7 @@
         <v>74</v>
       </c>
       <c r="C30" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="D30" t="s">
         <v>85</v>
@@ -2656,7 +2667,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="14" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>5</v>
       </c>
@@ -2685,7 +2696,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>5</v>
       </c>
@@ -2714,7 +2725,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>5</v>
       </c>
@@ -2743,7 +2754,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>5</v>
       </c>
@@ -2772,7 +2783,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>5</v>
       </c>
@@ -2795,7 +2806,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>5</v>
       </c>
@@ -2803,7 +2814,7 @@
         <v>283</v>
       </c>
       <c r="C36" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D36" t="s">
         <v>103</v>
@@ -2812,13 +2823,13 @@
         <v>6</v>
       </c>
       <c r="G36" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H36" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>5</v>
       </c>
@@ -2826,7 +2837,7 @@
         <v>876</v>
       </c>
       <c r="C37" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="D37" t="s">
         <v>103</v>
@@ -2835,13 +2846,13 @@
         <v>6</v>
       </c>
       <c r="G37" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H37" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>5</v>
       </c>
@@ -2870,7 +2881,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>5</v>
       </c>
@@ -2899,7 +2910,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>5</v>
       </c>
@@ -2928,7 +2939,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>5</v>
       </c>
@@ -2951,13 +2962,13 @@
         <v>369</v>
       </c>
       <c r="I41" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="J41" s="5" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>5</v>
       </c>
@@ -2983,7 +2994,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>5</v>
       </c>
@@ -3012,7 +3023,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>5</v>
       </c>
@@ -3041,7 +3052,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>5</v>
       </c>
@@ -3070,7 +3081,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>5</v>
       </c>
@@ -3096,7 +3107,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>5</v>
       </c>
@@ -3104,7 +3115,7 @@
         <v>23</v>
       </c>
       <c r="C47" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D47" t="s">
         <v>112</v>
@@ -3116,7 +3127,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>5</v>
       </c>
@@ -3124,7 +3135,7 @@
         <v>25</v>
       </c>
       <c r="C48" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="D48" t="s">
         <v>112</v>
@@ -3136,7 +3147,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
         <v>5</v>
       </c>
@@ -3153,7 +3164,7 @@
         <v>6</v>
       </c>
       <c r="F49" s="8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G49" s="7" t="s">
         <v>370</v>
@@ -3166,7 +3177,7 @@
       </c>
       <c r="J49" s="9"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>5</v>
       </c>
@@ -3195,7 +3206,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>5</v>
       </c>
@@ -3224,7 +3235,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>5</v>
       </c>
@@ -3253,7 +3264,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>5</v>
       </c>
@@ -3282,7 +3293,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>5</v>
       </c>
@@ -3311,7 +3322,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>5</v>
       </c>
@@ -3340,7 +3351,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="56" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="10" t="s">
         <v>5</v>
       </c>
@@ -3366,13 +3377,13 @@
         <v>369</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="J56" s="12" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="57" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="10" t="s">
         <v>5</v>
       </c>
@@ -3398,11 +3409,11 @@
         <v>369</v>
       </c>
       <c r="I57" s="10" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="J57" s="12"/>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>5</v>
       </c>
@@ -3431,7 +3442,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>5</v>
       </c>
@@ -3457,7 +3468,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>5</v>
       </c>
@@ -3486,7 +3497,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>5</v>
       </c>
@@ -3515,7 +3526,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>5</v>
       </c>
@@ -3535,7 +3546,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>5</v>
       </c>
@@ -3555,7 +3566,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>5</v>
       </c>
@@ -3584,7 +3595,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>5</v>
       </c>
@@ -3613,7 +3624,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>5</v>
       </c>
@@ -3630,7 +3641,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>5</v>
       </c>
@@ -3659,7 +3670,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>5</v>
       </c>
@@ -3688,7 +3699,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="69" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="10" t="s">
         <v>5</v>
       </c>
@@ -3714,13 +3725,13 @@
         <v>369</v>
       </c>
       <c r="I69" s="10" t="s">
+        <v>403</v>
+      </c>
+      <c r="J69" s="12" t="s">
         <v>404</v>
       </c>
-      <c r="J69" s="12" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" s="7" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="70" spans="1:10" s="7" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>5</v>
       </c>
@@ -3737,7 +3748,7 @@
         <v>17</v>
       </c>
       <c r="F70" s="8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G70" s="7" t="s">
         <v>370</v>
@@ -3746,13 +3757,13 @@
         <v>369</v>
       </c>
       <c r="I70" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="J70" s="9" t="s">
         <v>408</v>
       </c>
-      <c r="J70" s="9" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="71" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>5</v>
       </c>
@@ -3760,7 +3771,7 @@
         <v>378</v>
       </c>
       <c r="C71" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="D71" t="s">
         <v>168</v>
@@ -3770,17 +3781,17 @@
       </c>
       <c r="F71"/>
       <c r="G71" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H71" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="I71" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="J71"/>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>5</v>
       </c>
@@ -3809,7 +3820,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>5</v>
       </c>
@@ -3838,7 +3849,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="74" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="10" t="s">
         <v>5</v>
       </c>
@@ -3846,7 +3857,7 @@
         <v>23</v>
       </c>
       <c r="C74" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D74" s="10" t="s">
         <v>168</v>
@@ -3858,19 +3869,19 @@
         <v>2</v>
       </c>
       <c r="G74" s="10" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H74" s="10" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="I74" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="J74" s="12" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>5</v>
       </c>
@@ -3893,7 +3904,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="76" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="10" t="s">
         <v>5</v>
       </c>
@@ -3919,13 +3930,13 @@
         <v>369</v>
       </c>
       <c r="I76" s="10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J76" s="12" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="77" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="10" t="s">
         <v>5</v>
       </c>
@@ -3945,19 +3956,19 @@
         <v>3</v>
       </c>
       <c r="G77" s="10" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="H77" s="10" t="s">
         <v>369</v>
       </c>
       <c r="I77" s="10" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="J77" s="12" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>5</v>
       </c>
@@ -3986,7 +3997,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>5</v>
       </c>
@@ -4015,7 +4026,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>5</v>
       </c>
@@ -4044,7 +4055,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>5</v>
       </c>
@@ -4070,7 +4081,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="82" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="10" t="s">
         <v>5</v>
       </c>
@@ -4102,7 +4113,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="83" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="10" t="s">
         <v>5</v>
       </c>
@@ -4132,7 +4143,7 @@
       </c>
       <c r="J83" s="12"/>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>5</v>
       </c>
@@ -4152,7 +4163,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="85" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="10" t="s">
         <v>5</v>
       </c>
@@ -4178,13 +4189,13 @@
         <v>369</v>
       </c>
       <c r="I85" s="10" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="J85" s="12" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>5</v>
       </c>
@@ -4213,7 +4224,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>5</v>
       </c>
@@ -4242,7 +4253,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>5</v>
       </c>
@@ -4271,7 +4282,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>5</v>
       </c>
@@ -4300,7 +4311,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>5</v>
       </c>
@@ -4326,7 +4337,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="91" spans="1:10" s="10" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:10" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A91" s="10" t="s">
         <v>5</v>
       </c>
@@ -4352,13 +4363,13 @@
         <v>369</v>
       </c>
       <c r="I91" s="10" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="J91" s="12" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="10" t="s">
         <v>5</v>
       </c>
@@ -4384,13 +4395,13 @@
         <v>369</v>
       </c>
       <c r="I92" s="10" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="J92" s="12" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>5</v>
       </c>
@@ -4419,7 +4430,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>5</v>
       </c>
@@ -4448,7 +4459,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>5</v>
       </c>
@@ -4477,7 +4488,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>321</v>
       </c>
@@ -4506,7 +4517,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="97" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="10" t="s">
         <v>5</v>
       </c>
@@ -4529,16 +4540,16 @@
         <v>370</v>
       </c>
       <c r="H97" s="10" t="s">
+        <v>386</v>
+      </c>
+      <c r="I97" s="10" t="s">
         <v>387</v>
       </c>
-      <c r="I97" s="10" t="s">
+      <c r="J97" s="12" t="s">
         <v>388</v>
       </c>
-      <c r="J97" s="12" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>5</v>
       </c>
@@ -4558,7 +4569,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="99" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>5</v>
       </c>
@@ -4587,7 +4598,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>5</v>
       </c>
@@ -4616,7 +4627,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>5</v>
       </c>
@@ -4636,7 +4647,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>5</v>
       </c>
@@ -4656,10 +4667,10 @@
         <v>370</v>
       </c>
       <c r="H102" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="103" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>5</v>
       </c>
@@ -4688,7 +4699,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="104" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="10" t="s">
         <v>5</v>
       </c>
@@ -4696,7 +4707,7 @@
         <v>725</v>
       </c>
       <c r="C104" s="10" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D104" s="10" t="s">
         <v>203</v>
@@ -4708,19 +4719,19 @@
         <v>2</v>
       </c>
       <c r="G104" s="10" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H104" s="10" t="s">
+        <v>386</v>
+      </c>
+      <c r="I104" s="10" t="s">
         <v>387</v>
       </c>
-      <c r="I104" s="10" t="s">
+      <c r="J104" s="12" t="s">
         <v>388</v>
       </c>
-      <c r="J104" s="12" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="105" spans="1:10" s="10" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="105" spans="1:10" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A105" s="10" t="s">
         <v>5</v>
       </c>
@@ -4728,7 +4739,7 @@
         <v>773</v>
       </c>
       <c r="C105" s="10" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D105" s="10" t="s">
         <v>203</v>
@@ -4740,19 +4751,19 @@
         <v>2</v>
       </c>
       <c r="G105" s="10" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H105" s="10" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="I105" s="10" t="s">
+        <v>391</v>
+      </c>
+      <c r="J105" s="12" t="s">
         <v>392</v>
       </c>
-      <c r="J105" s="12" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="106" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="106" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="10" t="s">
         <v>5</v>
       </c>
@@ -4760,7 +4771,7 @@
         <v>444</v>
       </c>
       <c r="C106" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D106" s="10" t="s">
         <v>203</v>
@@ -4772,27 +4783,27 @@
         <v>2</v>
       </c>
       <c r="G106" s="10" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H106" s="10" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="I106" s="10" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J106" s="12" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="107" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="10" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B107" s="10" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C107" s="10" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D107" s="10" t="s">
         <v>203</v>
@@ -4804,27 +4815,27 @@
         <v>3</v>
       </c>
       <c r="G107" s="10" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H107" s="10" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="I107" s="10" t="s">
+        <v>395</v>
+      </c>
+      <c r="J107" s="12" t="s">
         <v>396</v>
       </c>
-      <c r="J107" s="12" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="108" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="108" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="10" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B108" s="10" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C108" s="10" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="D108" s="10" t="s">
         <v>203</v>
@@ -4836,19 +4847,19 @@
         <v>2</v>
       </c>
       <c r="G108" s="10" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H108" s="10" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="I108" s="10" t="s">
+        <v>400</v>
+      </c>
+      <c r="J108" s="12" t="s">
         <v>401</v>
       </c>
-      <c r="J108" s="12" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>5</v>
       </c>
@@ -4867,7 +4878,7 @@
       <c r="F109"/>
       <c r="J109"/>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>5</v>
       </c>
@@ -4896,7 +4907,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="111" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="10" t="s">
         <v>5</v>
       </c>
@@ -4922,13 +4933,13 @@
         <v>369</v>
       </c>
       <c r="I111" s="10" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="J111" s="12" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="112" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="10" t="s">
         <v>5</v>
       </c>
@@ -4954,13 +4965,13 @@
         <v>369</v>
       </c>
       <c r="I112" s="10" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="J112" s="12" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>5</v>
       </c>
@@ -4989,7 +5000,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>5</v>
       </c>
@@ -5018,7 +5029,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>5</v>
       </c>
@@ -5044,7 +5055,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="116" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="10" t="s">
         <v>5</v>
       </c>
@@ -5055,7 +5066,7 @@
         <v>262</v>
       </c>
       <c r="D116" s="10" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E116" s="10" t="s">
         <v>17</v>
@@ -5070,13 +5081,13 @@
         <v>369</v>
       </c>
       <c r="I116" s="10" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="J116" s="12" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="117" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="10" t="s">
         <v>5</v>
       </c>
@@ -5087,7 +5098,7 @@
         <v>263</v>
       </c>
       <c r="D117" s="10" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E117" s="10" t="s">
         <v>17</v>
@@ -5102,13 +5113,13 @@
         <v>369</v>
       </c>
       <c r="I117" s="10" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="J117" s="12" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>5</v>
       </c>
@@ -5137,7 +5148,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="119" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="10" t="s">
         <v>5</v>
       </c>
@@ -5148,7 +5159,7 @@
         <v>269</v>
       </c>
       <c r="D119" s="10" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E119" s="10" t="s">
         <v>17</v>
@@ -5163,13 +5174,13 @@
         <v>369</v>
       </c>
       <c r="I119" s="10" t="s">
+        <v>373</v>
+      </c>
+      <c r="J119" s="12" t="s">
         <v>374</v>
       </c>
-      <c r="J119" s="12" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>5</v>
       </c>
@@ -5192,13 +5203,13 @@
         <v>369</v>
       </c>
       <c r="I120" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="J120" s="5" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>5</v>
       </c>
@@ -5224,7 +5235,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>5</v>
       </c>
@@ -5250,7 +5261,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>5</v>
       </c>
@@ -5276,7 +5287,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>5</v>
       </c>
@@ -5305,7 +5316,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>5</v>
       </c>
@@ -5334,7 +5345,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>5</v>
       </c>
@@ -5363,7 +5374,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="127" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="10" t="s">
         <v>5</v>
       </c>
@@ -5371,7 +5382,7 @@
         <v>221</v>
       </c>
       <c r="C127" s="10" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D127" s="10" t="s">
         <v>248</v>
@@ -5383,17 +5394,17 @@
         <v>2</v>
       </c>
       <c r="G127" s="10" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="H127" s="10" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="I127" s="10" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="J127" s="12"/>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>5</v>
       </c>
@@ -5422,7 +5433,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>5</v>
       </c>
@@ -5442,7 +5453,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>5</v>
       </c>
@@ -5462,7 +5473,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>5</v>
       </c>
@@ -5482,7 +5493,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>5</v>
       </c>
@@ -5502,7 +5513,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>5</v>
       </c>
@@ -5522,7 +5533,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>5</v>
       </c>
@@ -5548,7 +5559,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>5</v>
       </c>
@@ -5574,7 +5585,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>5</v>
       </c>
@@ -5603,7 +5614,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>5</v>
       </c>
@@ -5629,7 +5640,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>5</v>
       </c>
@@ -5658,7 +5669,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>5</v>
       </c>
@@ -5684,7 +5695,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>5</v>
       </c>
@@ -5710,7 +5721,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>5</v>
       </c>
@@ -5739,7 +5750,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>5</v>
       </c>
@@ -5750,7 +5761,7 @@
         <v>313</v>
       </c>
       <c r="D142" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E142" t="s">
         <v>17</v>
@@ -5765,7 +5776,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>5</v>
       </c>
@@ -5776,7 +5787,7 @@
         <v>314</v>
       </c>
       <c r="D143" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E143" t="s">
         <v>17</v>
@@ -5791,7 +5802,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>5</v>
       </c>
@@ -5802,7 +5813,7 @@
         <v>315</v>
       </c>
       <c r="D144" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E144" t="s">
         <v>17</v>
@@ -5817,7 +5828,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>321</v>
       </c>
@@ -5828,7 +5839,7 @@
         <v>316</v>
       </c>
       <c r="D145" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E145" t="s">
         <v>17</v>
@@ -5846,7 +5857,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>321</v>
       </c>
@@ -5857,7 +5868,7 @@
         <v>317</v>
       </c>
       <c r="D146" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E146" t="s">
         <v>17</v>
@@ -5875,7 +5886,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>5</v>
       </c>
@@ -5886,7 +5897,7 @@
         <v>318</v>
       </c>
       <c r="D147" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E147" t="s">
         <v>47</v>
@@ -5895,7 +5906,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>5</v>
       </c>
@@ -5924,7 +5935,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>5</v>
       </c>
@@ -5953,7 +5964,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>5</v>
       </c>
@@ -5982,7 +5993,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>5</v>
       </c>
@@ -6008,7 +6019,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>5</v>
       </c>
@@ -6034,7 +6045,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>5</v>
       </c>
@@ -6063,7 +6074,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>5</v>
       </c>
@@ -6092,7 +6103,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>5</v>
       </c>
@@ -6121,7 +6132,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>5</v>
       </c>
@@ -6150,7 +6161,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>5</v>
       </c>
@@ -6179,7 +6190,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>5</v>
       </c>
@@ -6208,7 +6219,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>5</v>
       </c>
@@ -6237,7 +6248,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>5</v>
       </c>
@@ -6266,7 +6277,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>5</v>
       </c>
@@ -6292,7 +6303,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>5</v>
       </c>
@@ -6330,52 +6341,2019 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63392036-0DF4-41BC-932A-0EBA4F02E5CB}">
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:H188"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.1796875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.140625" style="14" customWidth="1"/>
+    <col min="6" max="6" width="21.42578125" customWidth="1"/>
+    <col min="7" max="7" width="22.85546875" customWidth="1"/>
+    <col min="8" max="8" width="46.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="E1" s="13" t="s">
         <v>367</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>365</v>
+      </c>
       <c r="G1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>365</v>
-      </c>
-      <c r="I1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>20</v>
       </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>17</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="4">
+        <v>1</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G2" s="15">
+        <v>46235</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>18</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="4">
+        <v>1</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G3" s="15">
+        <v>46235</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>19</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="4">
+        <v>20</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="4">
+        <v>21</v>
+      </c>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="4">
+        <v>22</v>
+      </c>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>23</v>
+      </c>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="4">
+        <v>24</v>
+      </c>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>25</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>26</v>
+      </c>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>27</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>28</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>29</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>30</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>31</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="4">
+        <v>32</v>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
+        <v>33</v>
+      </c>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="4">
+        <v>34</v>
+      </c>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="4">
+        <v>35</v>
+      </c>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="4">
+        <v>36</v>
+      </c>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="4">
+        <v>37</v>
+      </c>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="4">
+        <v>38</v>
+      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="4">
+        <v>39</v>
+      </c>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="4">
+        <v>40</v>
+      </c>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="4">
+        <v>41</v>
+      </c>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="4">
+        <v>42</v>
+      </c>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="4">
+        <v>43</v>
+      </c>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="4">
+        <v>44</v>
+      </c>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="4">
+        <v>45</v>
+      </c>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="4">
+        <v>46</v>
+      </c>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="4">
+        <v>47</v>
+      </c>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="4">
+        <v>48</v>
+      </c>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="4">
+        <v>49</v>
+      </c>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="4">
+        <v>50</v>
+      </c>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="4">
+        <v>51</v>
+      </c>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="4">
+        <v>52</v>
+      </c>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="4">
+        <v>53</v>
+      </c>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="4">
+        <v>54</v>
+      </c>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="4">
+        <v>55</v>
+      </c>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="4">
+        <v>56</v>
+      </c>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="4">
+        <v>57</v>
+      </c>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="4">
+        <v>58</v>
+      </c>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="4"/>
+      <c r="E43" s="4"/>
+      <c r="F43" s="4"/>
+      <c r="G43" s="4"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="4">
+        <v>59</v>
+      </c>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="4"/>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="4">
+        <v>60</v>
+      </c>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="4">
+        <v>61</v>
+      </c>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="4">
+        <v>62</v>
+      </c>
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="4"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="4">
+        <v>63</v>
+      </c>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="4">
+        <v>64</v>
+      </c>
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+      <c r="G49" s="4"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="4">
+        <v>65</v>
+      </c>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="4"/>
+      <c r="F50" s="4"/>
+      <c r="G50" s="4"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="4">
+        <v>66</v>
+      </c>
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4"/>
+      <c r="G51" s="4"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="4">
+        <v>67</v>
+      </c>
+      <c r="B52" s="4"/>
+      <c r="C52" s="4"/>
+      <c r="D52" s="4"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" s="4">
+        <v>68</v>
+      </c>
+      <c r="B53" s="4"/>
+      <c r="C53" s="4"/>
+      <c r="D53" s="4"/>
+      <c r="E53" s="4"/>
+      <c r="F53" s="4"/>
+      <c r="G53" s="4"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" s="4">
+        <v>69</v>
+      </c>
+      <c r="B54" s="4"/>
+      <c r="C54" s="4"/>
+      <c r="D54" s="4"/>
+      <c r="E54" s="4"/>
+      <c r="F54" s="4"/>
+      <c r="G54" s="4"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="4">
+        <v>70</v>
+      </c>
+      <c r="B55" s="4"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="4"/>
+      <c r="F55" s="4"/>
+      <c r="G55" s="4"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="4">
+        <v>71</v>
+      </c>
+      <c r="B56" s="4"/>
+      <c r="C56" s="4"/>
+      <c r="D56" s="4"/>
+      <c r="E56" s="4"/>
+      <c r="F56" s="4"/>
+      <c r="G56" s="4"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="4">
+        <v>72</v>
+      </c>
+      <c r="B57" s="4"/>
+      <c r="C57" s="4"/>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4"/>
+      <c r="F57" s="4"/>
+      <c r="G57" s="4"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="4">
+        <v>73</v>
+      </c>
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4"/>
+      <c r="G58" s="4"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="4">
+        <v>74</v>
+      </c>
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4"/>
+      <c r="E59" s="4"/>
+      <c r="F59" s="4"/>
+      <c r="G59" s="4"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="4">
+        <v>75</v>
+      </c>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="4"/>
+      <c r="F60" s="4"/>
+      <c r="G60" s="4"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" s="4">
+        <v>76</v>
+      </c>
+      <c r="B61" s="4"/>
+      <c r="C61" s="4"/>
+      <c r="D61" s="4"/>
+      <c r="E61" s="4"/>
+      <c r="F61" s="4"/>
+      <c r="G61" s="4"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" s="4">
+        <v>77</v>
+      </c>
+      <c r="B62" s="4"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="G62" s="4"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" s="4">
+        <v>78</v>
+      </c>
+      <c r="B63" s="4"/>
+      <c r="C63" s="4"/>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4"/>
+      <c r="G63" s="4"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" s="4">
+        <v>79</v>
+      </c>
+      <c r="B64" s="4"/>
+      <c r="C64" s="4"/>
+      <c r="D64" s="4"/>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4"/>
+      <c r="G64" s="4"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65" s="4">
+        <v>80</v>
+      </c>
+      <c r="B65" s="4"/>
+      <c r="C65" s="4"/>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
+      <c r="F65" s="4"/>
+      <c r="G65" s="4"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A66" s="4">
+        <v>81</v>
+      </c>
+      <c r="B66" s="4"/>
+      <c r="C66" s="4"/>
+      <c r="D66" s="4"/>
+      <c r="E66" s="4"/>
+      <c r="F66" s="4"/>
+      <c r="G66" s="4"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A67" s="4">
+        <v>82</v>
+      </c>
+      <c r="B67" s="4"/>
+      <c r="C67" s="4"/>
+      <c r="D67" s="4"/>
+      <c r="E67" s="4"/>
+      <c r="F67" s="4"/>
+      <c r="G67" s="4"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" s="4">
+        <v>83</v>
+      </c>
+      <c r="B68" s="4"/>
+      <c r="C68" s="4"/>
+      <c r="D68" s="4"/>
+      <c r="E68" s="4"/>
+      <c r="F68" s="4"/>
+      <c r="G68" s="4"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69" s="4">
+        <v>84</v>
+      </c>
+      <c r="B69" s="4"/>
+      <c r="C69" s="4"/>
+      <c r="D69" s="4"/>
+      <c r="E69" s="4"/>
+      <c r="F69" s="4"/>
+      <c r="G69" s="4"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70" s="4">
+        <v>85</v>
+      </c>
+      <c r="B70" s="4"/>
+      <c r="C70" s="4"/>
+      <c r="D70" s="4"/>
+      <c r="E70" s="4"/>
+      <c r="F70" s="4"/>
+      <c r="G70" s="4"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" s="4">
+        <v>86</v>
+      </c>
+      <c r="B71" s="4"/>
+      <c r="C71" s="4"/>
+      <c r="D71" s="4"/>
+      <c r="E71" s="4"/>
+      <c r="F71" s="4"/>
+      <c r="G71" s="4"/>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72" s="4">
+        <v>87</v>
+      </c>
+      <c r="B72" s="4"/>
+      <c r="C72" s="4"/>
+      <c r="D72" s="4"/>
+      <c r="E72" s="4"/>
+      <c r="F72" s="4"/>
+      <c r="G72" s="4"/>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A73" s="4">
+        <v>88</v>
+      </c>
+      <c r="B73" s="4"/>
+      <c r="C73" s="4"/>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+      <c r="F73" s="4"/>
+      <c r="G73" s="4"/>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A74" s="4">
+        <v>89</v>
+      </c>
+      <c r="B74" s="4"/>
+      <c r="C74" s="4"/>
+      <c r="D74" s="4"/>
+      <c r="E74" s="4"/>
+      <c r="F74" s="4"/>
+      <c r="G74" s="4"/>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A75" s="4">
+        <v>90</v>
+      </c>
+      <c r="B75" s="4"/>
+      <c r="C75" s="4"/>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4"/>
+      <c r="F75" s="4"/>
+      <c r="G75" s="4"/>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A76" s="4">
+        <v>91</v>
+      </c>
+      <c r="B76" s="4"/>
+      <c r="C76" s="4"/>
+      <c r="D76" s="4"/>
+      <c r="E76" s="4"/>
+      <c r="F76" s="4"/>
+      <c r="G76" s="4"/>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A77" s="4">
+        <v>92</v>
+      </c>
+      <c r="B77" s="4"/>
+      <c r="C77" s="4"/>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4"/>
+      <c r="F77" s="4"/>
+      <c r="G77" s="4"/>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A78" s="4">
+        <v>93</v>
+      </c>
+      <c r="B78" s="4"/>
+      <c r="C78" s="4"/>
+      <c r="D78" s="4"/>
+      <c r="E78" s="4"/>
+      <c r="F78" s="4"/>
+      <c r="G78" s="4"/>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A79" s="4">
+        <v>94</v>
+      </c>
+      <c r="B79" s="4"/>
+      <c r="C79" s="4"/>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4"/>
+      <c r="F79" s="4"/>
+      <c r="G79" s="4"/>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A80" s="4">
+        <v>95</v>
+      </c>
+      <c r="B80" s="4"/>
+      <c r="C80" s="4"/>
+      <c r="D80" s="4"/>
+      <c r="E80" s="4"/>
+      <c r="F80" s="4"/>
+      <c r="G80" s="4"/>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A81" s="4">
+        <v>96</v>
+      </c>
+      <c r="B81" s="4"/>
+      <c r="C81" s="4"/>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4"/>
+      <c r="F81" s="4"/>
+      <c r="G81" s="4"/>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A82" s="4">
+        <v>97</v>
+      </c>
+      <c r="B82" s="4"/>
+      <c r="C82" s="4"/>
+      <c r="D82" s="4"/>
+      <c r="E82" s="4"/>
+      <c r="F82" s="4"/>
+      <c r="G82" s="4"/>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A83" s="4">
+        <v>98</v>
+      </c>
+      <c r="B83" s="4"/>
+      <c r="C83" s="4"/>
+      <c r="D83" s="4"/>
+      <c r="E83" s="4"/>
+      <c r="F83" s="4"/>
+      <c r="G83" s="4"/>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A84" s="4">
+        <v>99</v>
+      </c>
+      <c r="B84" s="4"/>
+      <c r="C84" s="4"/>
+      <c r="D84" s="4"/>
+      <c r="E84" s="4"/>
+      <c r="F84" s="4"/>
+      <c r="G84" s="4"/>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A85" s="4">
+        <v>100</v>
+      </c>
+      <c r="B85" s="4"/>
+      <c r="C85" s="4"/>
+      <c r="D85" s="4"/>
+      <c r="E85" s="4"/>
+      <c r="F85" s="4"/>
+      <c r="G85" s="4"/>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A86" s="4">
+        <v>101</v>
+      </c>
+      <c r="B86" s="4"/>
+      <c r="C86" s="4"/>
+      <c r="D86" s="4"/>
+      <c r="E86" s="4"/>
+      <c r="F86" s="4"/>
+      <c r="G86" s="4"/>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A87" s="4">
+        <v>102</v>
+      </c>
+      <c r="B87" s="4"/>
+      <c r="C87" s="4"/>
+      <c r="D87" s="4"/>
+      <c r="E87" s="4"/>
+      <c r="F87" s="4"/>
+      <c r="G87" s="4"/>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A88" s="4">
+        <v>103</v>
+      </c>
+      <c r="B88" s="4"/>
+      <c r="C88" s="4"/>
+      <c r="D88" s="4"/>
+      <c r="E88" s="4"/>
+      <c r="F88" s="4"/>
+      <c r="G88" s="4"/>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A89" s="4">
+        <v>104</v>
+      </c>
+      <c r="B89" s="4"/>
+      <c r="C89" s="4"/>
+      <c r="D89" s="4"/>
+      <c r="E89" s="4"/>
+      <c r="F89" s="4"/>
+      <c r="G89" s="4"/>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A90" s="4">
+        <v>105</v>
+      </c>
+      <c r="B90" s="4"/>
+      <c r="C90" s="4"/>
+      <c r="D90" s="4"/>
+      <c r="E90" s="4"/>
+      <c r="F90" s="4"/>
+      <c r="G90" s="4"/>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A91" s="4">
+        <v>106</v>
+      </c>
+      <c r="B91" s="4"/>
+      <c r="C91" s="4"/>
+      <c r="D91" s="4"/>
+      <c r="E91" s="4"/>
+      <c r="F91" s="4"/>
+      <c r="G91" s="4"/>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A92" s="4">
+        <v>107</v>
+      </c>
+      <c r="B92" s="4"/>
+      <c r="C92" s="4"/>
+      <c r="D92" s="4"/>
+      <c r="E92" s="4"/>
+      <c r="F92" s="4"/>
+      <c r="G92" s="4"/>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A93" s="4">
+        <v>108</v>
+      </c>
+      <c r="B93" s="4"/>
+      <c r="C93" s="4"/>
+      <c r="D93" s="4"/>
+      <c r="E93" s="4"/>
+      <c r="F93" s="4"/>
+      <c r="G93" s="4"/>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A94" s="4">
+        <v>109</v>
+      </c>
+      <c r="B94" s="4"/>
+      <c r="C94" s="4"/>
+      <c r="D94" s="4"/>
+      <c r="E94" s="4"/>
+      <c r="F94" s="4"/>
+      <c r="G94" s="4"/>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A95" s="4">
+        <v>110</v>
+      </c>
+      <c r="B95" s="4"/>
+      <c r="C95" s="4"/>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4"/>
+      <c r="F95" s="4"/>
+      <c r="G95" s="4"/>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A96" s="4">
+        <v>111</v>
+      </c>
+      <c r="B96" s="4"/>
+      <c r="C96" s="4"/>
+      <c r="D96" s="4"/>
+      <c r="E96" s="4"/>
+      <c r="F96" s="4"/>
+      <c r="G96" s="4"/>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A97" s="4">
+        <v>112</v>
+      </c>
+      <c r="B97" s="4"/>
+      <c r="C97" s="4"/>
+      <c r="D97" s="4"/>
+      <c r="E97" s="4"/>
+      <c r="F97" s="4"/>
+      <c r="G97" s="4"/>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A98" s="4">
+        <v>113</v>
+      </c>
+      <c r="B98" s="4"/>
+      <c r="C98" s="4"/>
+      <c r="D98" s="4"/>
+      <c r="E98" s="4"/>
+      <c r="F98" s="4"/>
+      <c r="G98" s="4"/>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A99" s="4">
+        <v>114</v>
+      </c>
+      <c r="B99" s="4"/>
+      <c r="C99" s="4"/>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4"/>
+      <c r="F99" s="4"/>
+      <c r="G99" s="4"/>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A100" s="4">
+        <v>115</v>
+      </c>
+      <c r="B100" s="4"/>
+      <c r="C100" s="4"/>
+      <c r="D100" s="4"/>
+      <c r="E100" s="4"/>
+      <c r="F100" s="4"/>
+      <c r="G100" s="4"/>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A101" s="4">
+        <v>116</v>
+      </c>
+      <c r="B101" s="4"/>
+      <c r="C101" s="4"/>
+      <c r="D101" s="4"/>
+      <c r="E101" s="4"/>
+      <c r="F101" s="4"/>
+      <c r="G101" s="4"/>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A102" s="4">
+        <v>117</v>
+      </c>
+      <c r="B102" s="4"/>
+      <c r="C102" s="4"/>
+      <c r="D102" s="4"/>
+      <c r="E102" s="4"/>
+      <c r="F102" s="4"/>
+      <c r="G102" s="4"/>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A103" s="4">
+        <v>118</v>
+      </c>
+      <c r="B103" s="4"/>
+      <c r="C103" s="4"/>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4"/>
+      <c r="F103" s="4"/>
+      <c r="G103" s="4"/>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A104" s="4">
+        <v>119</v>
+      </c>
+      <c r="B104" s="4"/>
+      <c r="C104" s="4"/>
+      <c r="D104" s="4"/>
+      <c r="E104" s="4"/>
+      <c r="F104" s="4"/>
+      <c r="G104" s="4"/>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A105" s="4">
+        <v>120</v>
+      </c>
+      <c r="B105" s="4"/>
+      <c r="C105" s="4"/>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4"/>
+      <c r="F105" s="4"/>
+      <c r="G105" s="4"/>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A106" s="4">
+        <v>121</v>
+      </c>
+      <c r="B106" s="4"/>
+      <c r="C106" s="4"/>
+      <c r="D106" s="4"/>
+      <c r="E106" s="4"/>
+      <c r="F106" s="4"/>
+      <c r="G106" s="4"/>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A107" s="4">
+        <v>122</v>
+      </c>
+      <c r="B107" s="4"/>
+      <c r="C107" s="4"/>
+      <c r="D107" s="4"/>
+      <c r="E107" s="4"/>
+      <c r="F107" s="4"/>
+      <c r="G107" s="4"/>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A108" s="4">
+        <v>123</v>
+      </c>
+      <c r="B108" s="4"/>
+      <c r="C108" s="4"/>
+      <c r="D108" s="4"/>
+      <c r="E108" s="4"/>
+      <c r="F108" s="4"/>
+      <c r="G108" s="4"/>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A109" s="4">
+        <v>124</v>
+      </c>
+      <c r="B109" s="4"/>
+      <c r="C109" s="4"/>
+      <c r="D109" s="4"/>
+      <c r="E109" s="4"/>
+      <c r="F109" s="4"/>
+      <c r="G109" s="4"/>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A110" s="4">
+        <v>125</v>
+      </c>
+      <c r="B110" s="4"/>
+      <c r="C110" s="4"/>
+      <c r="D110" s="4"/>
+      <c r="E110" s="4"/>
+      <c r="F110" s="4"/>
+      <c r="G110" s="4"/>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A111" s="4">
+        <v>126</v>
+      </c>
+      <c r="B111" s="4"/>
+      <c r="C111" s="4"/>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4"/>
+      <c r="G111" s="4"/>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A112" s="4">
+        <v>127</v>
+      </c>
+      <c r="B112" s="4"/>
+      <c r="C112" s="4"/>
+      <c r="D112" s="4"/>
+      <c r="E112" s="4"/>
+      <c r="F112" s="4"/>
+      <c r="G112" s="4"/>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A113" s="4">
+        <v>128</v>
+      </c>
+      <c r="B113" s="4"/>
+      <c r="C113" s="4"/>
+      <c r="D113" s="4"/>
+      <c r="E113" s="4"/>
+      <c r="F113" s="4"/>
+      <c r="G113" s="4"/>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A114" s="4">
+        <v>129</v>
+      </c>
+      <c r="B114" s="4"/>
+      <c r="C114" s="4"/>
+      <c r="D114" s="4"/>
+      <c r="E114" s="4"/>
+      <c r="F114" s="4"/>
+      <c r="G114" s="4"/>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A115" s="4">
+        <v>130</v>
+      </c>
+      <c r="B115" s="4"/>
+      <c r="C115" s="4"/>
+      <c r="D115" s="4"/>
+      <c r="E115" s="4"/>
+      <c r="F115" s="4"/>
+      <c r="G115" s="4"/>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A116" s="4">
+        <v>131</v>
+      </c>
+      <c r="B116" s="4"/>
+      <c r="C116" s="4"/>
+      <c r="D116" s="4"/>
+      <c r="E116" s="4"/>
+      <c r="F116" s="4"/>
+      <c r="G116" s="4"/>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A117" s="4">
+        <v>132</v>
+      </c>
+      <c r="B117" s="4"/>
+      <c r="C117" s="4"/>
+      <c r="D117" s="4"/>
+      <c r="E117" s="4"/>
+      <c r="F117" s="4"/>
+      <c r="G117" s="4"/>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A118" s="4">
+        <v>133</v>
+      </c>
+      <c r="B118" s="4"/>
+      <c r="C118" s="4"/>
+      <c r="D118" s="4"/>
+      <c r="E118" s="4"/>
+      <c r="F118" s="4"/>
+      <c r="G118" s="4"/>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A119" s="4">
+        <v>134</v>
+      </c>
+      <c r="B119" s="4"/>
+      <c r="C119" s="4"/>
+      <c r="D119" s="4"/>
+      <c r="E119" s="4"/>
+      <c r="F119" s="4"/>
+      <c r="G119" s="4"/>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A120" s="4">
+        <v>135</v>
+      </c>
+      <c r="B120" s="4"/>
+      <c r="C120" s="4"/>
+      <c r="D120" s="4"/>
+      <c r="E120" s="4"/>
+      <c r="F120" s="4"/>
+      <c r="G120" s="4"/>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A121" s="4">
+        <v>136</v>
+      </c>
+      <c r="B121" s="4"/>
+      <c r="C121" s="4"/>
+      <c r="D121" s="4"/>
+      <c r="E121" s="4"/>
+      <c r="F121" s="4"/>
+      <c r="G121" s="4"/>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A122" s="4">
+        <v>137</v>
+      </c>
+      <c r="B122" s="4"/>
+      <c r="C122" s="4"/>
+      <c r="D122" s="4"/>
+      <c r="E122" s="4"/>
+      <c r="F122" s="4"/>
+      <c r="G122" s="4"/>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A123" s="4">
+        <v>138</v>
+      </c>
+      <c r="B123" s="4"/>
+      <c r="C123" s="4"/>
+      <c r="D123" s="4"/>
+      <c r="E123" s="4"/>
+      <c r="F123" s="4"/>
+      <c r="G123" s="4"/>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A124" s="4">
+        <v>139</v>
+      </c>
+      <c r="B124" s="4"/>
+      <c r="C124" s="4"/>
+      <c r="D124" s="4"/>
+      <c r="E124" s="4"/>
+      <c r="F124" s="4"/>
+      <c r="G124" s="4"/>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A125" s="4">
+        <v>140</v>
+      </c>
+      <c r="B125" s="4"/>
+      <c r="C125" s="4"/>
+      <c r="D125" s="4"/>
+      <c r="E125" s="4"/>
+      <c r="F125" s="4"/>
+      <c r="G125" s="4"/>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A126" s="4">
+        <v>141</v>
+      </c>
+      <c r="B126" s="4"/>
+      <c r="C126" s="4"/>
+      <c r="D126" s="4"/>
+      <c r="E126" s="4"/>
+      <c r="F126" s="4"/>
+      <c r="G126" s="4"/>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A127" s="4">
+        <v>142</v>
+      </c>
+      <c r="B127" s="4"/>
+      <c r="C127" s="4"/>
+      <c r="D127" s="4"/>
+      <c r="E127" s="4"/>
+      <c r="F127" s="4"/>
+      <c r="G127" s="4"/>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A128" s="4">
+        <v>143</v>
+      </c>
+      <c r="B128" s="4"/>
+      <c r="C128" s="4"/>
+      <c r="D128" s="4"/>
+      <c r="E128" s="4"/>
+      <c r="F128" s="4"/>
+      <c r="G128" s="4"/>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A129" s="4">
+        <v>144</v>
+      </c>
+      <c r="B129" s="4"/>
+      <c r="C129" s="4"/>
+      <c r="D129" s="4"/>
+      <c r="E129" s="4"/>
+      <c r="F129" s="4"/>
+      <c r="G129" s="4"/>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A130" s="4">
+        <v>145</v>
+      </c>
+      <c r="B130" s="4"/>
+      <c r="C130" s="4"/>
+      <c r="D130" s="4"/>
+      <c r="E130" s="4"/>
+      <c r="F130" s="4"/>
+      <c r="G130" s="4"/>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A131" s="4">
+        <v>146</v>
+      </c>
+      <c r="B131" s="4"/>
+      <c r="C131" s="4"/>
+      <c r="D131" s="4"/>
+      <c r="E131" s="4"/>
+      <c r="F131" s="4"/>
+      <c r="G131" s="4"/>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A132" s="4">
+        <v>147</v>
+      </c>
+      <c r="B132" s="4"/>
+      <c r="C132" s="4"/>
+      <c r="D132" s="4"/>
+      <c r="E132" s="4"/>
+      <c r="F132" s="4"/>
+      <c r="G132" s="4"/>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A133" s="4">
+        <v>148</v>
+      </c>
+      <c r="B133" s="4"/>
+      <c r="C133" s="4"/>
+      <c r="D133" s="4"/>
+      <c r="E133" s="4"/>
+      <c r="F133" s="4"/>
+      <c r="G133" s="4"/>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A134" s="4">
+        <v>149</v>
+      </c>
+      <c r="B134" s="4"/>
+      <c r="C134" s="4"/>
+      <c r="D134" s="4"/>
+      <c r="E134" s="4"/>
+      <c r="F134" s="4"/>
+      <c r="G134" s="4"/>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A135" s="4">
+        <v>150</v>
+      </c>
+      <c r="B135" s="4"/>
+      <c r="C135" s="4"/>
+      <c r="D135" s="4"/>
+      <c r="E135" s="4"/>
+      <c r="F135" s="4"/>
+      <c r="G135" s="4"/>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A136" s="4"/>
+      <c r="B136" s="4"/>
+      <c r="C136" s="4"/>
+      <c r="D136" s="4"/>
+      <c r="E136" s="4"/>
+      <c r="F136" s="4"/>
+      <c r="G136" s="4"/>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A137" s="4"/>
+      <c r="B137" s="4"/>
+      <c r="C137" s="4"/>
+      <c r="D137" s="4"/>
+      <c r="E137" s="4"/>
+      <c r="F137" s="4"/>
+      <c r="G137" s="4"/>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A138" s="4"/>
+      <c r="B138" s="4"/>
+      <c r="C138" s="4"/>
+      <c r="D138" s="4"/>
+      <c r="E138" s="4"/>
+      <c r="F138" s="4"/>
+      <c r="G138" s="4"/>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A139" s="4"/>
+      <c r="B139" s="4"/>
+      <c r="C139" s="4"/>
+      <c r="D139" s="4"/>
+      <c r="E139" s="4"/>
+      <c r="F139" s="4"/>
+      <c r="G139" s="4"/>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A140" s="4"/>
+      <c r="B140" s="4"/>
+      <c r="C140" s="4"/>
+      <c r="D140" s="4"/>
+      <c r="E140" s="4"/>
+      <c r="F140" s="4"/>
+      <c r="G140" s="4"/>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A141" s="4"/>
+      <c r="B141" s="4"/>
+      <c r="C141" s="4"/>
+      <c r="D141" s="4"/>
+      <c r="E141" s="4"/>
+      <c r="F141" s="4"/>
+      <c r="G141" s="4"/>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A142" s="4"/>
+      <c r="B142" s="4"/>
+      <c r="C142" s="4"/>
+      <c r="D142" s="4"/>
+      <c r="E142" s="4"/>
+      <c r="F142" s="4"/>
+      <c r="G142" s="4"/>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A143" s="4"/>
+      <c r="B143" s="4"/>
+      <c r="C143" s="4"/>
+      <c r="D143" s="4"/>
+      <c r="E143" s="4"/>
+      <c r="F143" s="4"/>
+      <c r="G143" s="4"/>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A144" s="4"/>
+      <c r="B144" s="4"/>
+      <c r="C144" s="4"/>
+      <c r="D144" s="4"/>
+      <c r="E144" s="4"/>
+      <c r="F144" s="4"/>
+      <c r="G144" s="4"/>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A145" s="4"/>
+      <c r="B145" s="4"/>
+      <c r="C145" s="4"/>
+      <c r="D145" s="4"/>
+      <c r="E145" s="4"/>
+      <c r="F145" s="4"/>
+      <c r="G145" s="4"/>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A146" s="4"/>
+      <c r="B146" s="4"/>
+      <c r="C146" s="4"/>
+      <c r="D146" s="4"/>
+      <c r="E146" s="4"/>
+      <c r="F146" s="4"/>
+      <c r="G146" s="4"/>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A147" s="4"/>
+      <c r="B147" s="4"/>
+      <c r="C147" s="4"/>
+      <c r="D147" s="4"/>
+      <c r="E147" s="4"/>
+      <c r="F147" s="4"/>
+      <c r="G147" s="4"/>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A148" s="4"/>
+      <c r="B148" s="4"/>
+      <c r="C148" s="4"/>
+      <c r="D148" s="4"/>
+      <c r="E148" s="4"/>
+      <c r="F148" s="4"/>
+      <c r="G148" s="4"/>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A149" s="4"/>
+      <c r="B149" s="4"/>
+      <c r="C149" s="4"/>
+      <c r="D149" s="4"/>
+      <c r="E149" s="4"/>
+      <c r="F149" s="4"/>
+      <c r="G149" s="4"/>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A150" s="4"/>
+      <c r="B150" s="4"/>
+      <c r="C150" s="4"/>
+      <c r="D150" s="4"/>
+      <c r="E150" s="4"/>
+      <c r="F150" s="4"/>
+      <c r="G150" s="4"/>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A151" s="4"/>
+      <c r="B151" s="4"/>
+      <c r="C151" s="4"/>
+      <c r="D151" s="4"/>
+      <c r="E151" s="4"/>
+      <c r="F151" s="4"/>
+      <c r="G151" s="4"/>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A152" s="4"/>
+      <c r="B152" s="4"/>
+      <c r="C152" s="4"/>
+      <c r="D152" s="4"/>
+      <c r="E152" s="4"/>
+      <c r="F152" s="4"/>
+      <c r="G152" s="4"/>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A153" s="4"/>
+      <c r="B153" s="4"/>
+      <c r="C153" s="4"/>
+      <c r="D153" s="4"/>
+      <c r="E153" s="4"/>
+      <c r="F153" s="4"/>
+      <c r="G153" s="4"/>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" s="4"/>
+      <c r="B154" s="4"/>
+      <c r="C154" s="4"/>
+      <c r="D154" s="4"/>
+      <c r="E154" s="4"/>
+      <c r="F154" s="4"/>
+      <c r="G154" s="4"/>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A155" s="4"/>
+      <c r="B155" s="4"/>
+      <c r="C155" s="4"/>
+      <c r="D155" s="4"/>
+      <c r="E155" s="4"/>
+      <c r="F155" s="4"/>
+      <c r="G155" s="4"/>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A156" s="4"/>
+      <c r="B156" s="4"/>
+      <c r="C156" s="4"/>
+      <c r="D156" s="4"/>
+      <c r="E156" s="4"/>
+      <c r="F156" s="4"/>
+      <c r="G156" s="4"/>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A157" s="4"/>
+      <c r="B157" s="4"/>
+      <c r="C157" s="4"/>
+      <c r="D157" s="4"/>
+      <c r="E157" s="4"/>
+      <c r="F157" s="4"/>
+      <c r="G157" s="4"/>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A158" s="4"/>
+      <c r="B158" s="4"/>
+      <c r="C158" s="4"/>
+      <c r="D158" s="4"/>
+      <c r="E158" s="4"/>
+      <c r="F158" s="4"/>
+      <c r="G158" s="4"/>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A159" s="4"/>
+      <c r="B159" s="4"/>
+      <c r="C159" s="4"/>
+      <c r="D159" s="4"/>
+      <c r="E159" s="4"/>
+      <c r="F159" s="4"/>
+      <c r="G159" s="4"/>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A160" s="4"/>
+      <c r="B160" s="4"/>
+      <c r="C160" s="4"/>
+      <c r="D160" s="4"/>
+      <c r="E160" s="4"/>
+      <c r="F160" s="4"/>
+      <c r="G160" s="4"/>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A161" s="4"/>
+      <c r="B161" s="4"/>
+      <c r="C161" s="4"/>
+      <c r="D161" s="4"/>
+      <c r="E161" s="4"/>
+      <c r="F161" s="4"/>
+      <c r="G161" s="4"/>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A162" s="4"/>
+      <c r="B162" s="4"/>
+      <c r="C162" s="4"/>
+      <c r="D162" s="4"/>
+      <c r="E162" s="4"/>
+      <c r="F162" s="4"/>
+      <c r="G162" s="4"/>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A163" s="4"/>
+      <c r="B163" s="4"/>
+      <c r="C163" s="4"/>
+      <c r="D163" s="4"/>
+      <c r="E163" s="4"/>
+      <c r="F163" s="4"/>
+      <c r="G163" s="4"/>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A164" s="4"/>
+      <c r="B164" s="4"/>
+      <c r="C164" s="4"/>
+      <c r="D164" s="4"/>
+      <c r="E164" s="4"/>
+      <c r="F164" s="4"/>
+      <c r="G164" s="4"/>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A165" s="4"/>
+      <c r="B165" s="4"/>
+      <c r="C165" s="4"/>
+      <c r="D165" s="4"/>
+      <c r="E165" s="4"/>
+      <c r="F165" s="4"/>
+      <c r="G165" s="4"/>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A166" s="4"/>
+      <c r="B166" s="4"/>
+      <c r="C166" s="4"/>
+      <c r="D166" s="4"/>
+      <c r="E166" s="4"/>
+      <c r="F166" s="4"/>
+      <c r="G166" s="4"/>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A167" s="4"/>
+      <c r="B167" s="4"/>
+      <c r="C167" s="4"/>
+      <c r="D167" s="4"/>
+      <c r="E167" s="4"/>
+      <c r="F167" s="4"/>
+      <c r="G167" s="4"/>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A168" s="4"/>
+      <c r="B168" s="4"/>
+      <c r="C168" s="4"/>
+      <c r="D168" s="4"/>
+      <c r="E168" s="4"/>
+      <c r="F168" s="4"/>
+      <c r="G168" s="4"/>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A169" s="4"/>
+      <c r="B169" s="4"/>
+      <c r="C169" s="4"/>
+      <c r="D169" s="4"/>
+      <c r="E169" s="4"/>
+      <c r="F169" s="4"/>
+      <c r="G169" s="4"/>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A170" s="4"/>
+      <c r="B170" s="4"/>
+      <c r="C170" s="4"/>
+      <c r="D170" s="4"/>
+      <c r="E170" s="4"/>
+      <c r="F170" s="4"/>
+      <c r="G170" s="4"/>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A171" s="4"/>
+      <c r="B171" s="4"/>
+      <c r="C171" s="4"/>
+      <c r="D171" s="4"/>
+      <c r="E171" s="4"/>
+      <c r="F171" s="4"/>
+      <c r="G171" s="4"/>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A172" s="4"/>
+      <c r="B172" s="4"/>
+      <c r="C172" s="4"/>
+      <c r="D172" s="4"/>
+      <c r="E172" s="4"/>
+      <c r="F172" s="4"/>
+      <c r="G172" s="4"/>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A173" s="4"/>
+      <c r="B173" s="4"/>
+      <c r="C173" s="4"/>
+      <c r="D173" s="4"/>
+      <c r="E173" s="4"/>
+      <c r="F173" s="4"/>
+      <c r="G173" s="4"/>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A174" s="4"/>
+      <c r="B174" s="4"/>
+      <c r="C174" s="4"/>
+      <c r="D174" s="4"/>
+      <c r="E174" s="4"/>
+      <c r="F174" s="4"/>
+      <c r="G174" s="4"/>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A175" s="4"/>
+      <c r="B175" s="4"/>
+      <c r="C175" s="4"/>
+      <c r="D175" s="4"/>
+      <c r="E175" s="4"/>
+      <c r="F175" s="4"/>
+      <c r="G175" s="4"/>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A176" s="4"/>
+      <c r="B176" s="4"/>
+      <c r="C176" s="4"/>
+      <c r="D176" s="4"/>
+      <c r="E176" s="4"/>
+      <c r="F176" s="4"/>
+      <c r="G176" s="4"/>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A177" s="4"/>
+      <c r="B177" s="4"/>
+      <c r="C177" s="4"/>
+      <c r="D177" s="4"/>
+      <c r="E177" s="4"/>
+      <c r="F177" s="4"/>
+      <c r="G177" s="4"/>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A178" s="4"/>
+      <c r="B178" s="4"/>
+      <c r="C178" s="4"/>
+      <c r="D178" s="4"/>
+      <c r="E178" s="4"/>
+      <c r="F178" s="4"/>
+      <c r="G178" s="4"/>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A179" s="4"/>
+      <c r="B179" s="4"/>
+      <c r="C179" s="4"/>
+      <c r="D179" s="4"/>
+      <c r="E179" s="4"/>
+      <c r="F179" s="4"/>
+      <c r="G179" s="4"/>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A180" s="4"/>
+      <c r="B180" s="4"/>
+      <c r="C180" s="4"/>
+      <c r="D180" s="4"/>
+      <c r="E180" s="4"/>
+      <c r="F180" s="4"/>
+      <c r="G180" s="4"/>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A181" s="4"/>
+      <c r="B181" s="4"/>
+      <c r="C181" s="4"/>
+      <c r="D181" s="4"/>
+      <c r="E181" s="4"/>
+      <c r="F181" s="4"/>
+      <c r="G181" s="4"/>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A182" s="4"/>
+      <c r="B182" s="4"/>
+      <c r="C182" s="4"/>
+      <c r="D182" s="4"/>
+      <c r="E182" s="4"/>
+      <c r="F182" s="4"/>
+      <c r="G182" s="4"/>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A183" s="4"/>
+      <c r="B183" s="4"/>
+      <c r="C183" s="4"/>
+      <c r="D183" s="4"/>
+      <c r="E183" s="4"/>
+      <c r="F183" s="4"/>
+      <c r="G183" s="4"/>
+    </row>
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A184" s="4"/>
+      <c r="B184" s="4"/>
+      <c r="C184" s="4"/>
+      <c r="D184" s="4"/>
+      <c r="E184" s="4"/>
+      <c r="F184" s="4"/>
+      <c r="G184" s="4"/>
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A185" s="4"/>
+      <c r="B185" s="4"/>
+      <c r="C185" s="4"/>
+      <c r="D185" s="4"/>
+      <c r="E185" s="4"/>
+      <c r="F185" s="4"/>
+      <c r="G185" s="4"/>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A186" s="4"/>
+      <c r="B186" s="4"/>
+      <c r="C186" s="4"/>
+      <c r="D186" s="4"/>
+      <c r="E186" s="4"/>
+      <c r="F186" s="4"/>
+      <c r="G186" s="4"/>
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A187" s="4"/>
+      <c r="B187" s="4"/>
+      <c r="C187" s="4"/>
+      <c r="D187" s="4"/>
+      <c r="E187" s="4"/>
+      <c r="F187" s="4"/>
+      <c r="G187" s="4"/>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A188" s="4"/>
+      <c r="B188" s="4"/>
+      <c r="C188" s="4"/>
+      <c r="D188" s="4"/>
+      <c r="E188" s="4"/>
+      <c r="F188" s="4"/>
+      <c r="G188" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
structy sliding window challenges
</commit_message>
<xml_diff>
--- a/docs/Programming Puzzles.xlsx
+++ b/docs/Programming Puzzles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\ProjectDSA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD9A901F-6090-4E21-BF3F-C185C0E7C9CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF741154-FE47-4DA3-96C5-75D3C879CC90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1228" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1281" uniqueCount="442">
   <si>
     <t>PLATFORM</t>
   </si>
@@ -1308,6 +1308,63 @@
   </si>
   <si>
     <t>In Rating 1 - 5: 1 being very easy, 5 being very hard.</t>
+  </si>
+  <si>
+    <t>Longest Unique Substring</t>
+  </si>
+  <si>
+    <t>Longest Subarray Sum</t>
+  </si>
+  <si>
+    <t>Find Subarray Sum</t>
+  </si>
+  <si>
+    <t>Count Substring Anagrams</t>
+  </si>
+  <si>
+    <t>Has Substring Anagram</t>
+  </si>
+  <si>
+    <t>Subarray Target Sum Size K</t>
+  </si>
+  <si>
+    <t>Max Subarray Sum Size K</t>
+  </si>
+  <si>
+    <t>Max Subarray Product Size K</t>
+  </si>
+  <si>
+    <t>Graph</t>
+  </si>
+  <si>
+    <t>Prereqs Possible</t>
+  </si>
+  <si>
+    <t>27/09/2026</t>
+  </si>
+  <si>
+    <t>01/08/2026</t>
+  </si>
+  <si>
+    <t>Longest Two Char Substring</t>
+  </si>
+  <si>
+    <t>Max Ones With Single Flip</t>
+  </si>
+  <si>
+    <t>Count Subarray Product</t>
+  </si>
+  <si>
+    <t>Count Substring At Most K Distinct</t>
+  </si>
+  <si>
+    <t>Count Substring Exactly K Distinct</t>
+  </si>
+  <si>
+    <t>28/09/2026</t>
+  </si>
+  <si>
+    <t>Sliding Window with Variable Size Recipe</t>
   </si>
 </sst>
 </file>
@@ -1392,7 +1449,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1424,9 +1481,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="3" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -6341,16 +6396,16 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63392036-0DF4-41BC-932A-0EBA4F02E5CB}">
-  <dimension ref="A1:H188"/>
+  <dimension ref="A1:H182"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
     <col min="3" max="3" width="18.5703125" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.140625" style="14" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="19.140625" customWidth="1"/>
     <col min="6" max="6" width="21.42578125" customWidth="1"/>
-    <col min="7" max="7" width="22.85546875" customWidth="1"/>
+    <col min="7" max="7" width="24.42578125" customWidth="1"/>
     <col min="8" max="8" width="46.5703125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6367,7 +6422,7 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="1" t="s">
         <v>367</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -6399,8 +6454,8 @@
       <c r="F2" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="G2" s="15">
-        <v>46235</v>
+      <c r="G2" s="13" t="s">
+        <v>434</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -6422,8 +6477,8 @@
       <c r="F3" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="G3" s="15">
-        <v>46235</v>
+      <c r="G3" s="13" t="s">
+        <v>434</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -6435,7 +6490,7 @@
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
+      <c r="G4" s="13"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
@@ -6446,7 +6501,7 @@
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
+      <c r="G5" s="13"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
@@ -6457,7 +6512,7 @@
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
+      <c r="G6" s="13"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
@@ -6468,7 +6523,7 @@
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
+      <c r="G7" s="13"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
@@ -6479,7 +6534,7 @@
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
+      <c r="G8" s="13"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
@@ -6490,7 +6545,7 @@
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
+      <c r="G9" s="13"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
@@ -6501,7 +6556,7 @@
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
+      <c r="G10" s="13"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
@@ -6512,7 +6567,7 @@
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
+      <c r="G11" s="13"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
@@ -6523,7 +6578,7 @@
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
+      <c r="G12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
@@ -6534,7 +6589,7 @@
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
+      <c r="G13" s="13"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
@@ -6545,7 +6600,7 @@
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
+      <c r="G14" s="13"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
@@ -6556,7 +6611,7 @@
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
+      <c r="G15" s="13"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
@@ -6567,7 +6622,7 @@
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
+      <c r="G16" s="13"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
@@ -6578,7 +6633,7 @@
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
+      <c r="G17" s="13"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
@@ -6589,7 +6644,7 @@
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
+      <c r="G18" s="13"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
@@ -6600,7 +6655,7 @@
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
+      <c r="G19" s="13"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
@@ -6611,7 +6666,7 @@
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
+      <c r="G20" s="13"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
@@ -6622,7 +6677,7 @@
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
+      <c r="G21" s="13"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
@@ -6633,7 +6688,7 @@
       <c r="D22" s="4"/>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="G22" s="13"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
@@ -6644,7 +6699,7 @@
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
+      <c r="G23" s="13"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
@@ -6655,7 +6710,7 @@
       <c r="D24" s="4"/>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
+      <c r="G24" s="13"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
@@ -6666,7 +6721,7 @@
       <c r="D25" s="4"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
+      <c r="G25" s="13"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
@@ -6677,7 +6732,7 @@
       <c r="D26" s="4"/>
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
+      <c r="G26" s="13"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
@@ -6688,7 +6743,7 @@
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
+      <c r="G27" s="13"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
@@ -6699,7 +6754,7 @@
       <c r="D28" s="4"/>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
+      <c r="G28" s="13"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
@@ -6710,7 +6765,7 @@
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
+      <c r="G29" s="13"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
@@ -6721,7 +6776,7 @@
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
+      <c r="G30" s="13"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
@@ -6732,7 +6787,7 @@
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
+      <c r="G31" s="13"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
@@ -6743,7 +6798,7 @@
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
+      <c r="G32" s="13"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
@@ -6754,7 +6809,7 @@
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
+      <c r="G33" s="13"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
@@ -6765,7 +6820,7 @@
       <c r="D34" s="4"/>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
+      <c r="G34" s="13"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="4">
@@ -6776,7 +6831,7 @@
       <c r="D35" s="4"/>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
+      <c r="G35" s="13"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
@@ -6787,7 +6842,7 @@
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
       <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
+      <c r="G36" s="13"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="4">
@@ -6798,7 +6853,7 @@
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
       <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
+      <c r="G37" s="13"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="4">
@@ -6809,7 +6864,7 @@
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
+      <c r="G38" s="13"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="4">
@@ -6820,7 +6875,7 @@
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
+      <c r="G39" s="13"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="4">
@@ -6831,7 +6886,7 @@
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
-      <c r="G40" s="4"/>
+      <c r="G40" s="13"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="4">
@@ -6842,7 +6897,7 @@
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
+      <c r="G41" s="13"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="4">
@@ -6853,7 +6908,7 @@
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
+      <c r="G42" s="13"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="4">
@@ -6864,7 +6919,7 @@
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
-      <c r="G43" s="4"/>
+      <c r="G43" s="13"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="4">
@@ -6875,7 +6930,7 @@
       <c r="D44" s="4"/>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
-      <c r="G44" s="4"/>
+      <c r="G44" s="13"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="4">
@@ -6886,7 +6941,7 @@
       <c r="D45" s="4"/>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
+      <c r="G45" s="13"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="4">
@@ -6897,7 +6952,7 @@
       <c r="D46" s="4"/>
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
+      <c r="G46" s="13"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="4">
@@ -6908,7 +6963,7 @@
       <c r="D47" s="4"/>
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
+      <c r="G47" s="13"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="4">
@@ -6919,7 +6974,7 @@
       <c r="D48" s="4"/>
       <c r="E48" s="4"/>
       <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
+      <c r="G48" s="13"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="4">
@@ -6930,7 +6985,7 @@
       <c r="D49" s="4"/>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
+      <c r="G49" s="13"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="4">
@@ -6941,7 +6996,7 @@
       <c r="D50" s="4"/>
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
-      <c r="G50" s="4"/>
+      <c r="G50" s="13"/>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="4">
@@ -6952,7 +7007,7 @@
       <c r="D51" s="4"/>
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
+      <c r="G51" s="13"/>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="4">
@@ -6963,7 +7018,7 @@
       <c r="D52" s="4"/>
       <c r="E52" s="4"/>
       <c r="F52" s="4"/>
-      <c r="G52" s="4"/>
+      <c r="G52" s="13"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="4">
@@ -6974,7 +7029,7 @@
       <c r="D53" s="4"/>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
-      <c r="G53" s="4"/>
+      <c r="G53" s="13"/>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="4">
@@ -6985,7 +7040,7 @@
       <c r="D54" s="4"/>
       <c r="E54" s="4"/>
       <c r="F54" s="4"/>
-      <c r="G54" s="4"/>
+      <c r="G54" s="13"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="4">
@@ -6996,7 +7051,7 @@
       <c r="D55" s="4"/>
       <c r="E55" s="4"/>
       <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
+      <c r="G55" s="13"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="4">
@@ -7007,7 +7062,7 @@
       <c r="D56" s="4"/>
       <c r="E56" s="4"/>
       <c r="F56" s="4"/>
-      <c r="G56" s="4"/>
+      <c r="G56" s="13"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="4">
@@ -7018,7 +7073,7 @@
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
       <c r="F57" s="4"/>
-      <c r="G57" s="4"/>
+      <c r="G57" s="13"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="4">
@@ -7029,7 +7084,7 @@
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
       <c r="F58" s="4"/>
-      <c r="G58" s="4"/>
+      <c r="G58" s="13"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="4">
@@ -7040,7 +7095,7 @@
       <c r="D59" s="4"/>
       <c r="E59" s="4"/>
       <c r="F59" s="4"/>
-      <c r="G59" s="4"/>
+      <c r="G59" s="13"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="4">
@@ -7051,7 +7106,7 @@
       <c r="D60" s="4"/>
       <c r="E60" s="4"/>
       <c r="F60" s="4"/>
-      <c r="G60" s="4"/>
+      <c r="G60" s="13"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="4">
@@ -7062,7 +7117,7 @@
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
       <c r="F61" s="4"/>
-      <c r="G61" s="4"/>
+      <c r="G61" s="13"/>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="4">
@@ -7073,7 +7128,7 @@
       <c r="D62" s="4"/>
       <c r="E62" s="4"/>
       <c r="F62" s="4"/>
-      <c r="G62" s="4"/>
+      <c r="G62" s="13"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="4">
@@ -7084,7 +7139,7 @@
       <c r="D63" s="4"/>
       <c r="E63" s="4"/>
       <c r="F63" s="4"/>
-      <c r="G63" s="4"/>
+      <c r="G63" s="13"/>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="4">
@@ -7095,7 +7150,7 @@
       <c r="D64" s="4"/>
       <c r="E64" s="4"/>
       <c r="F64" s="4"/>
-      <c r="G64" s="4"/>
+      <c r="G64" s="13"/>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="4">
@@ -7106,7 +7161,7 @@
       <c r="D65" s="4"/>
       <c r="E65" s="4"/>
       <c r="F65" s="4"/>
-      <c r="G65" s="4"/>
+      <c r="G65" s="13"/>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="4">
@@ -7117,7 +7172,7 @@
       <c r="D66" s="4"/>
       <c r="E66" s="4"/>
       <c r="F66" s="4"/>
-      <c r="G66" s="4"/>
+      <c r="G66" s="13"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="4">
@@ -7128,7 +7183,7 @@
       <c r="D67" s="4"/>
       <c r="E67" s="4"/>
       <c r="F67" s="4"/>
-      <c r="G67" s="4"/>
+      <c r="G67" s="13"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
@@ -7139,7 +7194,7 @@
       <c r="D68" s="4"/>
       <c r="E68" s="4"/>
       <c r="F68" s="4"/>
-      <c r="G68" s="4"/>
+      <c r="G68" s="13"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="4">
@@ -7150,7 +7205,7 @@
       <c r="D69" s="4"/>
       <c r="E69" s="4"/>
       <c r="F69" s="4"/>
-      <c r="G69" s="4"/>
+      <c r="G69" s="13"/>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
@@ -7161,7 +7216,7 @@
       <c r="D70" s="4"/>
       <c r="E70" s="4"/>
       <c r="F70" s="4"/>
-      <c r="G70" s="4"/>
+      <c r="G70" s="13"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="4">
@@ -7172,7 +7227,7 @@
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
       <c r="F71" s="4"/>
-      <c r="G71" s="4"/>
+      <c r="G71" s="13"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="4">
@@ -7183,7 +7238,7 @@
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
       <c r="F72" s="4"/>
-      <c r="G72" s="4"/>
+      <c r="G72" s="13"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="4">
@@ -7194,7 +7249,7 @@
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>
       <c r="F73" s="4"/>
-      <c r="G73" s="4"/>
+      <c r="G73" s="13"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="4">
@@ -7205,7 +7260,7 @@
       <c r="D74" s="4"/>
       <c r="E74" s="4"/>
       <c r="F74" s="4"/>
-      <c r="G74" s="4"/>
+      <c r="G74" s="13"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="4">
@@ -7216,7 +7271,7 @@
       <c r="D75" s="4"/>
       <c r="E75" s="4"/>
       <c r="F75" s="4"/>
-      <c r="G75" s="4"/>
+      <c r="G75" s="13"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="4">
@@ -7227,7 +7282,7 @@
       <c r="D76" s="4"/>
       <c r="E76" s="4"/>
       <c r="F76" s="4"/>
-      <c r="G76" s="4"/>
+      <c r="G76" s="13"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="4">
@@ -7238,7 +7293,7 @@
       <c r="D77" s="4"/>
       <c r="E77" s="4"/>
       <c r="F77" s="4"/>
-      <c r="G77" s="4"/>
+      <c r="G77" s="13"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="4">
@@ -7249,7 +7304,7 @@
       <c r="D78" s="4"/>
       <c r="E78" s="4"/>
       <c r="F78" s="4"/>
-      <c r="G78" s="4"/>
+      <c r="G78" s="13"/>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="4">
@@ -7260,573 +7315,680 @@
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>
       <c r="F79" s="4"/>
-      <c r="G79" s="4"/>
+      <c r="G79" s="13"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
         <v>95</v>
       </c>
-      <c r="B80" s="4"/>
-      <c r="C80" s="4"/>
+      <c r="B80" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>431</v>
+      </c>
       <c r="D80" s="4"/>
       <c r="E80" s="4"/>
-      <c r="F80" s="4"/>
-      <c r="G80" s="4"/>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F80" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G80" s="13"/>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" s="4">
-        <v>96</v>
-      </c>
-      <c r="B81" s="4"/>
-      <c r="C81" s="4"/>
+        <v>99</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>231</v>
+      </c>
       <c r="D81" s="4"/>
       <c r="E81" s="4"/>
-      <c r="F81" s="4"/>
-      <c r="G81" s="4"/>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F81" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G81" s="13"/>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82" s="4">
-        <v>97</v>
-      </c>
-      <c r="B82" s="4"/>
-      <c r="C82" s="4"/>
+        <v>100</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>231</v>
+      </c>
       <c r="D82" s="4"/>
       <c r="E82" s="4"/>
-      <c r="F82" s="4"/>
-      <c r="G82" s="4"/>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F82" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G82" s="13"/>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="4">
-        <v>98</v>
-      </c>
-      <c r="B83" s="4"/>
-      <c r="C83" s="4"/>
+        <v>103</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>231</v>
+      </c>
       <c r="D83" s="4"/>
       <c r="E83" s="4"/>
-      <c r="F83" s="4"/>
-      <c r="G83" s="4"/>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F83" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G83" s="13"/>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" s="4">
-        <v>99</v>
-      </c>
-      <c r="B84" s="4"/>
-      <c r="C84" s="4"/>
+        <v>104</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>231</v>
+      </c>
       <c r="D84" s="4"/>
       <c r="E84" s="4"/>
-      <c r="F84" s="4"/>
-      <c r="G84" s="4"/>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F84" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G84" s="13"/>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" s="4">
-        <v>100</v>
-      </c>
-      <c r="B85" s="4"/>
-      <c r="C85" s="4"/>
+        <v>105</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>426</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>231</v>
+      </c>
       <c r="D85" s="4"/>
       <c r="E85" s="4"/>
-      <c r="F85" s="4"/>
-      <c r="G85" s="4"/>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F85" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G85" s="13"/>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" s="4">
-        <v>101</v>
-      </c>
-      <c r="B86" s="4"/>
-      <c r="C86" s="4"/>
+        <v>106</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>231</v>
+      </c>
       <c r="D86" s="4"/>
       <c r="E86" s="4"/>
-      <c r="F86" s="4"/>
-      <c r="G86" s="4"/>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F86" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G86" s="13"/>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87" s="4">
-        <v>102</v>
-      </c>
-      <c r="B87" s="4"/>
-      <c r="C87" s="4"/>
+        <v>107</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>231</v>
+      </c>
       <c r="D87" s="4"/>
       <c r="E87" s="4"/>
-      <c r="F87" s="4"/>
-      <c r="G87" s="4"/>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F87" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G87" s="13"/>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" s="4">
-        <v>103</v>
-      </c>
-      <c r="B88" s="4"/>
-      <c r="C88" s="4"/>
-      <c r="D88" s="4"/>
-      <c r="E88" s="4"/>
-      <c r="F88" s="4"/>
-      <c r="G88" s="4"/>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>423</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="D88" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E88" s="4">
+        <v>2</v>
+      </c>
+      <c r="F88" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G88" s="13" t="s">
+        <v>433</v>
+      </c>
+      <c r="H88" s="4" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89" s="4">
-        <v>104</v>
-      </c>
-      <c r="B89" s="4"/>
-      <c r="C89" s="4"/>
-      <c r="D89" s="4"/>
-      <c r="E89" s="4"/>
-      <c r="F89" s="4"/>
-      <c r="G89" s="4"/>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E89" s="4">
+        <v>2</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G89" s="13" t="s">
+        <v>440</v>
+      </c>
+      <c r="H89" s="4" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90" s="4">
-        <v>105</v>
-      </c>
-      <c r="B90" s="4"/>
-      <c r="C90" s="4"/>
-      <c r="D90" s="4"/>
-      <c r="E90" s="4"/>
-      <c r="F90" s="4"/>
-      <c r="G90" s="4"/>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E90" s="4">
+        <v>2</v>
+      </c>
+      <c r="F90" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G90" s="13" t="s">
+        <v>440</v>
+      </c>
+      <c r="H90" s="4" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91" s="4">
-        <v>106</v>
-      </c>
-      <c r="B91" s="4"/>
-      <c r="C91" s="4"/>
+        <v>112</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>231</v>
+      </c>
       <c r="D91" s="4"/>
       <c r="E91" s="4"/>
-      <c r="F91" s="4"/>
-      <c r="G91" s="4"/>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F91" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G91" s="13"/>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92" s="4">
-        <v>107</v>
-      </c>
-      <c r="B92" s="4"/>
-      <c r="C92" s="4"/>
+        <v>113</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>231</v>
+      </c>
       <c r="D92" s="4"/>
       <c r="E92" s="4"/>
-      <c r="F92" s="4"/>
-      <c r="G92" s="4"/>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F92" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G92" s="13"/>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93" s="4">
-        <v>108</v>
-      </c>
-      <c r="B93" s="4"/>
-      <c r="C93" s="4"/>
+        <v>114</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>231</v>
+      </c>
       <c r="D93" s="4"/>
       <c r="E93" s="4"/>
-      <c r="F93" s="4"/>
-      <c r="G93" s="4"/>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F93" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="G93" s="13"/>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94" s="4">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="B94" s="4"/>
       <c r="C94" s="4"/>
       <c r="D94" s="4"/>
       <c r="E94" s="4"/>
       <c r="F94" s="4"/>
-      <c r="G94" s="4"/>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G94" s="13"/>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95" s="4">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B95" s="4"/>
       <c r="C95" s="4"/>
       <c r="D95" s="4"/>
       <c r="E95" s="4"/>
       <c r="F95" s="4"/>
-      <c r="G95" s="4"/>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G95" s="13"/>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96" s="4">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="B96" s="4"/>
       <c r="C96" s="4"/>
       <c r="D96" s="4"/>
       <c r="E96" s="4"/>
       <c r="F96" s="4"/>
-      <c r="G96" s="4"/>
+      <c r="G96" s="13"/>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="4">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B97" s="4"/>
       <c r="C97" s="4"/>
       <c r="D97" s="4"/>
       <c r="E97" s="4"/>
       <c r="F97" s="4"/>
-      <c r="G97" s="4"/>
+      <c r="G97" s="13"/>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="4">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B98" s="4"/>
       <c r="C98" s="4"/>
       <c r="D98" s="4"/>
       <c r="E98" s="4"/>
       <c r="F98" s="4"/>
-      <c r="G98" s="4"/>
+      <c r="G98" s="13"/>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A99" s="4">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B99" s="4"/>
       <c r="C99" s="4"/>
       <c r="D99" s="4"/>
       <c r="E99" s="4"/>
       <c r="F99" s="4"/>
-      <c r="G99" s="4"/>
+      <c r="G99" s="13"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B100" s="4"/>
       <c r="C100" s="4"/>
       <c r="D100" s="4"/>
       <c r="E100" s="4"/>
       <c r="F100" s="4"/>
-      <c r="G100" s="4"/>
+      <c r="G100" s="13"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B101" s="4"/>
       <c r="C101" s="4"/>
       <c r="D101" s="4"/>
       <c r="E101" s="4"/>
       <c r="F101" s="4"/>
-      <c r="G101" s="4"/>
+      <c r="G101" s="13"/>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B102" s="4"/>
       <c r="C102" s="4"/>
       <c r="D102" s="4"/>
       <c r="E102" s="4"/>
       <c r="F102" s="4"/>
-      <c r="G102" s="4"/>
+      <c r="G102" s="13"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B103" s="4"/>
       <c r="C103" s="4"/>
       <c r="D103" s="4"/>
       <c r="E103" s="4"/>
       <c r="F103" s="4"/>
-      <c r="G103" s="4"/>
+      <c r="G103" s="13"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B104" s="4"/>
       <c r="C104" s="4"/>
       <c r="D104" s="4"/>
       <c r="E104" s="4"/>
       <c r="F104" s="4"/>
-      <c r="G104" s="4"/>
+      <c r="G104" s="13"/>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B105" s="4"/>
       <c r="C105" s="4"/>
       <c r="D105" s="4"/>
       <c r="E105" s="4"/>
       <c r="F105" s="4"/>
-      <c r="G105" s="4"/>
+      <c r="G105" s="13"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="4">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B106" s="4"/>
       <c r="C106" s="4"/>
       <c r="D106" s="4"/>
       <c r="E106" s="4"/>
       <c r="F106" s="4"/>
-      <c r="G106" s="4"/>
+      <c r="G106" s="13"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B107" s="4"/>
       <c r="C107" s="4"/>
       <c r="D107" s="4"/>
       <c r="E107" s="4"/>
       <c r="F107" s="4"/>
-      <c r="G107" s="4"/>
+      <c r="G107" s="13"/>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="B108" s="4"/>
       <c r="C108" s="4"/>
       <c r="D108" s="4"/>
       <c r="E108" s="4"/>
       <c r="F108" s="4"/>
-      <c r="G108" s="4"/>
+      <c r="G108" s="13"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B109" s="4"/>
       <c r="C109" s="4"/>
       <c r="D109" s="4"/>
       <c r="E109" s="4"/>
       <c r="F109" s="4"/>
-      <c r="G109" s="4"/>
+      <c r="G109" s="13"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B110" s="4"/>
       <c r="C110" s="4"/>
       <c r="D110" s="4"/>
       <c r="E110" s="4"/>
       <c r="F110" s="4"/>
-      <c r="G110" s="4"/>
+      <c r="G110" s="13"/>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B111" s="4"/>
       <c r="C111" s="4"/>
       <c r="D111" s="4"/>
       <c r="E111" s="4"/>
       <c r="F111" s="4"/>
-      <c r="G111" s="4"/>
+      <c r="G111" s="13"/>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B112" s="4"/>
       <c r="C112" s="4"/>
       <c r="D112" s="4"/>
       <c r="E112" s="4"/>
       <c r="F112" s="4"/>
-      <c r="G112" s="4"/>
+      <c r="G112" s="13"/>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" s="4">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B113" s="4"/>
       <c r="C113" s="4"/>
       <c r="D113" s="4"/>
       <c r="E113" s="4"/>
       <c r="F113" s="4"/>
-      <c r="G113" s="4"/>
+      <c r="G113" s="13"/>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A114" s="4">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B114" s="4"/>
       <c r="C114" s="4"/>
       <c r="D114" s="4"/>
       <c r="E114" s="4"/>
       <c r="F114" s="4"/>
-      <c r="G114" s="4"/>
+      <c r="G114" s="13"/>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" s="4">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B115" s="4"/>
       <c r="C115" s="4"/>
       <c r="D115" s="4"/>
       <c r="E115" s="4"/>
       <c r="F115" s="4"/>
-      <c r="G115" s="4"/>
+      <c r="G115" s="13"/>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" s="4">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B116" s="4"/>
       <c r="C116" s="4"/>
       <c r="D116" s="4"/>
       <c r="E116" s="4"/>
       <c r="F116" s="4"/>
-      <c r="G116" s="4"/>
+      <c r="G116" s="13"/>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" s="4">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B117" s="4"/>
       <c r="C117" s="4"/>
       <c r="D117" s="4"/>
       <c r="E117" s="4"/>
       <c r="F117" s="4"/>
-      <c r="G117" s="4"/>
+      <c r="G117" s="13"/>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" s="4">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B118" s="4"/>
       <c r="C118" s="4"/>
       <c r="D118" s="4"/>
       <c r="E118" s="4"/>
       <c r="F118" s="4"/>
-      <c r="G118" s="4"/>
+      <c r="G118" s="13"/>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" s="4">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B119" s="4"/>
       <c r="C119" s="4"/>
       <c r="D119" s="4"/>
       <c r="E119" s="4"/>
       <c r="F119" s="4"/>
-      <c r="G119" s="4"/>
+      <c r="G119" s="13"/>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A120" s="4">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B120" s="4"/>
       <c r="C120" s="4"/>
       <c r="D120" s="4"/>
       <c r="E120" s="4"/>
       <c r="F120" s="4"/>
-      <c r="G120" s="4"/>
+      <c r="G120" s="13"/>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A121" s="4">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B121" s="4"/>
       <c r="C121" s="4"/>
       <c r="D121" s="4"/>
       <c r="E121" s="4"/>
       <c r="F121" s="4"/>
-      <c r="G121" s="4"/>
+      <c r="G121" s="13"/>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A122" s="4">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B122" s="4"/>
       <c r="C122" s="4"/>
       <c r="D122" s="4"/>
       <c r="E122" s="4"/>
       <c r="F122" s="4"/>
-      <c r="G122" s="4"/>
+      <c r="G122" s="13"/>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A123" s="4">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B123" s="4"/>
       <c r="C123" s="4"/>
       <c r="D123" s="4"/>
       <c r="E123" s="4"/>
       <c r="F123" s="4"/>
-      <c r="G123" s="4"/>
+      <c r="G123" s="13"/>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B124" s="4"/>
       <c r="C124" s="4"/>
       <c r="D124" s="4"/>
       <c r="E124" s="4"/>
       <c r="F124" s="4"/>
-      <c r="G124" s="4"/>
+      <c r="G124" s="13"/>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A125" s="4">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="B125" s="4"/>
       <c r="C125" s="4"/>
       <c r="D125" s="4"/>
       <c r="E125" s="4"/>
       <c r="F125" s="4"/>
-      <c r="G125" s="4"/>
+      <c r="G125" s="13"/>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A126" s="4">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B126" s="4"/>
       <c r="C126" s="4"/>
       <c r="D126" s="4"/>
       <c r="E126" s="4"/>
       <c r="F126" s="4"/>
-      <c r="G126" s="4"/>
+      <c r="G126" s="13"/>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A127" s="4">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B127" s="4"/>
       <c r="C127" s="4"/>
       <c r="D127" s="4"/>
       <c r="E127" s="4"/>
       <c r="F127" s="4"/>
-      <c r="G127" s="4"/>
+      <c r="G127" s="13"/>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A128" s="4">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B128" s="4"/>
       <c r="C128" s="4"/>
       <c r="D128" s="4"/>
       <c r="E128" s="4"/>
       <c r="F128" s="4"/>
-      <c r="G128" s="4"/>
+      <c r="G128" s="13"/>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A129" s="4">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B129" s="4"/>
       <c r="C129" s="4"/>
       <c r="D129" s="4"/>
       <c r="E129" s="4"/>
       <c r="F129" s="4"/>
-      <c r="G129" s="4"/>
+      <c r="G129" s="13"/>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A130" s="4">
-        <v>145</v>
-      </c>
+      <c r="A130" s="4"/>
       <c r="B130" s="4"/>
       <c r="C130" s="4"/>
       <c r="D130" s="4"/>
       <c r="E130" s="4"/>
       <c r="F130" s="4"/>
-      <c r="G130" s="4"/>
+      <c r="G130" s="13"/>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A131" s="4">
-        <v>146</v>
-      </c>
+      <c r="A131" s="4"/>
       <c r="B131" s="4"/>
       <c r="C131" s="4"/>
       <c r="D131" s="4"/>
@@ -7835,9 +7997,7 @@
       <c r="G131" s="4"/>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A132" s="4">
-        <v>147</v>
-      </c>
+      <c r="A132" s="4"/>
       <c r="B132" s="4"/>
       <c r="C132" s="4"/>
       <c r="D132" s="4"/>
@@ -7846,9 +8006,7 @@
       <c r="G132" s="4"/>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A133" s="4">
-        <v>148</v>
-      </c>
+      <c r="A133" s="4"/>
       <c r="B133" s="4"/>
       <c r="C133" s="4"/>
       <c r="D133" s="4"/>
@@ -7857,9 +8015,7 @@
       <c r="G133" s="4"/>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A134" s="4">
-        <v>149</v>
-      </c>
+      <c r="A134" s="4"/>
       <c r="B134" s="4"/>
       <c r="C134" s="4"/>
       <c r="D134" s="4"/>
@@ -7868,9 +8024,7 @@
       <c r="G134" s="4"/>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A135" s="4">
-        <v>150</v>
-      </c>
+      <c r="A135" s="4"/>
       <c r="B135" s="4"/>
       <c r="C135" s="4"/>
       <c r="D135" s="4"/>
@@ -8301,60 +8455,6 @@
       <c r="F182" s="4"/>
       <c r="G182" s="4"/>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A183" s="4"/>
-      <c r="B183" s="4"/>
-      <c r="C183" s="4"/>
-      <c r="D183" s="4"/>
-      <c r="E183" s="4"/>
-      <c r="F183" s="4"/>
-      <c r="G183" s="4"/>
-    </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A184" s="4"/>
-      <c r="B184" s="4"/>
-      <c r="C184" s="4"/>
-      <c r="D184" s="4"/>
-      <c r="E184" s="4"/>
-      <c r="F184" s="4"/>
-      <c r="G184" s="4"/>
-    </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A185" s="4"/>
-      <c r="B185" s="4"/>
-      <c r="C185" s="4"/>
-      <c r="D185" s="4"/>
-      <c r="E185" s="4"/>
-      <c r="F185" s="4"/>
-      <c r="G185" s="4"/>
-    </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A186" s="4"/>
-      <c r="B186" s="4"/>
-      <c r="C186" s="4"/>
-      <c r="D186" s="4"/>
-      <c r="E186" s="4"/>
-      <c r="F186" s="4"/>
-      <c r="G186" s="4"/>
-    </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A187" s="4"/>
-      <c r="B187" s="4"/>
-      <c r="C187" s="4"/>
-      <c r="D187" s="4"/>
-      <c r="E187" s="4"/>
-      <c r="F187" s="4"/>
-      <c r="G187" s="4"/>
-    </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A188" s="4"/>
-      <c r="B188" s="4"/>
-      <c r="C188" s="4"/>
-      <c r="D188" s="4"/>
-      <c r="E188" s="4"/>
-      <c r="F188" s="4"/>
-      <c r="G188" s="4"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
structy two pointer challenges
</commit_message>
<xml_diff>
--- a/docs/Programming Puzzles.xlsx
+++ b/docs/Programming Puzzles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\ProjectDSA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B81EC1E-6FE4-4683-8C6F-AA090F0E26C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A30B7D-13E7-4081-9C0F-CABEA31C462B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1296" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1303" uniqueCount="451">
   <si>
     <t>PLATFORM</t>
   </si>
@@ -1383,6 +1383,15 @@
   </si>
   <si>
     <t>30/09/2026</t>
+  </si>
+  <si>
+    <t>Uncompress</t>
+  </si>
+  <si>
+    <t>Compress</t>
+  </si>
+  <si>
+    <t>Trick with appending special character.</t>
   </si>
 </sst>
 </file>
@@ -7576,25 +7585,44 @@
       <c r="A95" s="4">
         <v>118</v>
       </c>
-      <c r="B95" s="4"/>
+      <c r="B95" s="4" t="s">
+        <v>448</v>
+      </c>
       <c r="C95" s="4" t="s">
         <v>442</v>
       </c>
-      <c r="D95" s="4"/>
-      <c r="E95" s="4"/>
-      <c r="F95" s="13"/>
+      <c r="D95" s="4">
+        <v>2</v>
+      </c>
+      <c r="E95" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F95" s="13" t="s">
+        <v>447</v>
+      </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" s="4">
         <v>119</v>
       </c>
-      <c r="B96" s="4"/>
+      <c r="B96" s="4" t="s">
+        <v>449</v>
+      </c>
       <c r="C96" s="4" t="s">
         <v>442</v>
       </c>
-      <c r="D96" s="4"/>
-      <c r="E96" s="4"/>
-      <c r="F96" s="13"/>
+      <c r="D96" s="4">
+        <v>2</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F96" s="13" t="s">
+        <v>447</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>450</v>
+      </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" s="4">

</xml_diff>

<commit_message>
structy binary search challenges
</commit_message>
<xml_diff>
--- a/docs/Programming Puzzles.xlsx
+++ b/docs/Programming Puzzles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\ProjectDSA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F80EE6-C899-418B-947B-34BD6D9A9D8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E767B8E-085A-45C4-8593-17844FC95C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1313" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="461">
   <si>
     <t>PLATFORM</t>
   </si>
@@ -1404,6 +1404,24 @@
   </si>
   <si>
     <t>Is Subsequence</t>
+  </si>
+  <si>
+    <t>02/10/2026</t>
+  </si>
+  <si>
+    <t>Binary Search Index</t>
+  </si>
+  <si>
+    <t>Square Root</t>
+  </si>
+  <si>
+    <t>Trick: Right pointer is the answer if you cannot find it in the while loop. Equivalent to rounding down.</t>
+  </si>
+  <si>
+    <t>Trick: Left pointer is the answer if you cannot find it in the while loop.</t>
+  </si>
+  <si>
+    <t>Find Leftmost Index</t>
   </si>
 </sst>
 </file>
@@ -1863,7 +1881,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="65.140625" customWidth="1"/>
+    <col min="1" max="1" width="53.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -6435,7 +6453,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63392036-0DF4-41BC-932A-0EBA4F02E5CB}">
-  <dimension ref="A1:G178"/>
+  <dimension ref="A1:G177"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -7689,45 +7707,81 @@
       <c r="C99" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="D99" s="4"/>
+      <c r="D99" s="4">
+        <v>1</v>
+      </c>
       <c r="E99" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="F99" s="13"/>
+      <c r="F99" s="13" t="s">
+        <v>455</v>
+      </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A100" s="4">
         <v>125</v>
       </c>
-      <c r="B100" s="4"/>
-      <c r="C100" s="4"/>
-      <c r="D100" s="4"/>
-      <c r="E100" s="4"/>
-      <c r="F100" s="13"/>
+      <c r="B100" s="4" t="s">
+        <v>456</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D100" s="4">
+        <v>2</v>
+      </c>
+      <c r="E100" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F100" s="13" t="s">
+        <v>455</v>
+      </c>
+      <c r="G100" s="4" t="s">
+        <v>459</v>
+      </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A101" s="4">
         <v>126</v>
       </c>
-      <c r="B101" s="4"/>
-      <c r="C101" s="4"/>
-      <c r="D101" s="4"/>
-      <c r="E101" s="4"/>
-      <c r="F101" s="13"/>
+      <c r="B101" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D101" s="4">
+        <v>2</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F101" s="13" t="s">
+        <v>455</v>
+      </c>
+      <c r="G101" s="4" t="s">
+        <v>458</v>
+      </c>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A102" s="4">
-        <v>127</v>
-      </c>
-      <c r="B102" s="4"/>
-      <c r="C102" s="4"/>
+        <v>128</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>460</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>85</v>
+      </c>
       <c r="D102" s="4"/>
-      <c r="E102" s="4"/>
+      <c r="E102" s="4" t="s">
+        <v>366</v>
+      </c>
       <c r="F102" s="13"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A103" s="4">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B103" s="4"/>
       <c r="C103" s="4"/>
@@ -7737,7 +7791,7 @@
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A104" s="4">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B104" s="4"/>
       <c r="C104" s="4"/>
@@ -7747,7 +7801,7 @@
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A105" s="4">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B105" s="4"/>
       <c r="C105" s="4"/>
@@ -7757,7 +7811,7 @@
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A106" s="4">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B106" s="4"/>
       <c r="C106" s="4"/>
@@ -7767,7 +7821,7 @@
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A107" s="4">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B107" s="4"/>
       <c r="C107" s="4"/>
@@ -7777,7 +7831,7 @@
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A108" s="4">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B108" s="4"/>
       <c r="C108" s="4"/>
@@ -7787,7 +7841,7 @@
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B109" s="4"/>
       <c r="C109" s="4"/>
@@ -7797,7 +7851,7 @@
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B110" s="4"/>
       <c r="C110" s="4"/>
@@ -7807,7 +7861,7 @@
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="4">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B111" s="4"/>
       <c r="C111" s="4"/>
@@ -7817,7 +7871,7 @@
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A112" s="4">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B112" s="4"/>
       <c r="C112" s="4"/>
@@ -7827,7 +7881,7 @@
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" s="4">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B113" s="4"/>
       <c r="C113" s="4"/>
@@ -7837,7 +7891,7 @@
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" s="4">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B114" s="4"/>
       <c r="C114" s="4"/>
@@ -7847,7 +7901,7 @@
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" s="4">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B115" s="4"/>
       <c r="C115" s="4"/>
@@ -7857,7 +7911,7 @@
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" s="4">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B116" s="4"/>
       <c r="C116" s="4"/>
@@ -7867,7 +7921,7 @@
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" s="4">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B117" s="4"/>
       <c r="C117" s="4"/>
@@ -7877,7 +7931,7 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" s="4">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B118" s="4"/>
       <c r="C118" s="4"/>
@@ -7887,7 +7941,7 @@
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" s="4">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B119" s="4"/>
       <c r="C119" s="4"/>
@@ -7897,7 +7951,7 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" s="4">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B120" s="4"/>
       <c r="C120" s="4"/>
@@ -7907,7 +7961,7 @@
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" s="4">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B121" s="4"/>
       <c r="C121" s="4"/>
@@ -7917,7 +7971,7 @@
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" s="4">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B122" s="4"/>
       <c r="C122" s="4"/>
@@ -7927,7 +7981,7 @@
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" s="4">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B123" s="4"/>
       <c r="C123" s="4"/>
@@ -7937,7 +7991,7 @@
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" s="4">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B124" s="4"/>
       <c r="C124" s="4"/>
@@ -7946,9 +8000,7 @@
       <c r="F124" s="13"/>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A125" s="4">
-        <v>150</v>
-      </c>
+      <c r="A125" s="4"/>
       <c r="B125" s="4"/>
       <c r="C125" s="4"/>
       <c r="D125" s="4"/>
@@ -7961,7 +8013,7 @@
       <c r="C126" s="4"/>
       <c r="D126" s="4"/>
       <c r="E126" s="4"/>
-      <c r="F126" s="13"/>
+      <c r="F126" s="4"/>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" s="4"/>
@@ -8371,14 +8423,6 @@
       <c r="E177" s="4"/>
       <c r="F177" s="4"/>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A178" s="4"/>
-      <c r="B178" s="4"/>
-      <c r="C178" s="4"/>
-      <c r="D178" s="4"/>
-      <c r="E178" s="4"/>
-      <c r="F178" s="4"/>
-    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
structy dynamic programming challenges
</commit_message>
<xml_diff>
--- a/docs/Programming Puzzles.xlsx
+++ b/docs/Programming Puzzles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\ProjectDSA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{122714F2-376D-46CB-A97A-0726EF7EEBD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{456A8465-8BE0-424D-ABE1-8685508C11AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1356" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1367" uniqueCount="479">
   <si>
     <t>PLATFORM</t>
   </si>
@@ -1464,6 +1464,18 @@
   </si>
   <si>
     <t>Fibonacci</t>
+  </si>
+  <si>
+    <t>Memoization for the win. Brings it down from O(2^n) to O(n). Use hashmaps for constant time lookups.</t>
+  </si>
+  <si>
+    <t>Sum Possible</t>
+  </si>
+  <si>
+    <t>Tribonacci</t>
+  </si>
+  <si>
+    <t>It's so elegant :)</t>
   </si>
 </sst>
 </file>
@@ -7924,7 +7936,7 @@
         <v>366</v>
       </c>
       <c r="F106" s="15" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="G106" s="14" t="s">
         <v>472</v>
@@ -7947,7 +7959,7 @@
         <v>366</v>
       </c>
       <c r="F107" s="13" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="G107" s="4" t="s">
         <v>473</v>
@@ -7963,31 +7975,61 @@
       <c r="C108" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="D108" s="4"/>
+      <c r="D108" s="4">
+        <v>1</v>
+      </c>
       <c r="E108" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="F108" s="13"/>
+      <c r="F108" s="13" t="s">
+        <v>465</v>
+      </c>
+      <c r="G108" s="4" t="s">
+        <v>475</v>
+      </c>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A109" s="4">
         <v>138</v>
       </c>
-      <c r="B109" s="4"/>
-      <c r="C109" s="4"/>
-      <c r="D109" s="4"/>
-      <c r="E109" s="4"/>
-      <c r="F109" s="13"/>
+      <c r="B109" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="D109" s="4">
+        <v>1</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F109" s="13" t="s">
+        <v>465</v>
+      </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A110" s="4">
         <v>139</v>
       </c>
-      <c r="B110" s="4"/>
-      <c r="C110" s="4"/>
-      <c r="D110" s="4"/>
-      <c r="E110" s="4"/>
-      <c r="F110" s="13"/>
+      <c r="B110" s="4" t="s">
+        <v>476</v>
+      </c>
+      <c r="C110" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="D110" s="4">
+        <v>2</v>
+      </c>
+      <c r="E110" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F110" s="13" t="s">
+        <v>468</v>
+      </c>
+      <c r="G110" s="4" t="s">
+        <v>478</v>
+      </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A111" s="4">

</xml_diff>

<commit_message>
structy array and string challenges
</commit_message>
<xml_diff>
--- a/docs/Programming Puzzles.xlsx
+++ b/docs/Programming Puzzles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\ProjectDSA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50A0ACE4-4321-4D78-B7E4-07397754C469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61C869C2-76FB-45EB-B658-C9321B61174E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1714" uniqueCount="521">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1470" uniqueCount="524">
   <si>
     <t>PLATFORM</t>
   </si>
@@ -1602,6 +1602,15 @@
   </si>
   <si>
     <t>Tricky to come up with this stack solution that's why it's a 3. Easy pattern once you know what it is though.</t>
+  </si>
+  <si>
+    <t>Introduction to the Prefix Sum pattern.</t>
+  </si>
+  <si>
+    <t>Has Subarray Sum</t>
+  </si>
+  <si>
+    <t>I need to get used to the Prefix Sum pattern.</t>
   </si>
 </sst>
 </file>
@@ -6655,7 +6664,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63392036-0DF4-41BC-932A-0EBA4F02E5CB}">
-  <dimension ref="A1:G167"/>
+  <dimension ref="A1:G214"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -8616,21 +8625,41 @@
       <c r="C131" s="4" t="s">
         <v>519</v>
       </c>
-      <c r="D131" s="4"/>
+      <c r="D131" s="4">
+        <v>1</v>
+      </c>
       <c r="E131" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="F131" s="4"/>
+      <c r="F131" s="13" t="s">
+        <v>511</v>
+      </c>
+      <c r="G131" s="5" t="s">
+        <v>521</v>
+      </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A132" s="4">
         <v>168</v>
       </c>
-      <c r="B132" s="4"/>
-      <c r="C132" s="4"/>
-      <c r="D132" s="4"/>
-      <c r="E132" s="4"/>
-      <c r="F132" s="4"/>
+      <c r="B132" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="D132" s="4">
+        <v>2</v>
+      </c>
+      <c r="E132" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F132" s="13" t="s">
+        <v>511</v>
+      </c>
+      <c r="G132" s="5" t="s">
+        <v>523</v>
+      </c>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A133" s="4">
@@ -8953,7 +8982,9 @@
       <c r="F164" s="4"/>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A165" s="4"/>
+      <c r="A165" s="4">
+        <v>201</v>
+      </c>
       <c r="B165" s="4"/>
       <c r="C165" s="4"/>
       <c r="D165" s="4"/>
@@ -8961,7 +8992,9 @@
       <c r="F165" s="4"/>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A166" s="4"/>
+      <c r="A166" s="4">
+        <v>202</v>
+      </c>
       <c r="B166" s="4"/>
       <c r="C166" s="4"/>
       <c r="D166" s="4"/>
@@ -8969,13 +9002,250 @@
       <c r="F166" s="4"/>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A167" s="4"/>
+      <c r="A167" s="4">
+        <v>203</v>
+      </c>
       <c r="B167" s="4"/>
       <c r="C167" s="4"/>
       <c r="D167" s="4"/>
       <c r="E167" s="4"/>
       <c r="F167" s="4"/>
     </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A168" s="4">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A169" s="4">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A170" s="4">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A171" s="4">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A172" s="4">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A173" s="4">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A174" s="4">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A175" s="4">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A176" s="4">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A177" s="4">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A178" s="4">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A179" s="4">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A180" s="4">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A181" s="4">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A182" s="4">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A183" s="4">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A184" s="4">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A185" s="4">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A186" s="4">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A187" s="4">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A188" s="4">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A189" s="4">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A190" s="4">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A191" s="4">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A192" s="4">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A193" s="4">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A194" s="4">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A195" s="4">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A196" s="4">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A197" s="4">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A198" s="4">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A199" s="4">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A200" s="4">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A201" s="4">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A202" s="4">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A203" s="4">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A204" s="4">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="205" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A205" s="4">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="206" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A206" s="4">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="207" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A207" s="4">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="208" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A208" s="4">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A209" s="4">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="210" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A210" s="4">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="211" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A211" s="4">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="212" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A212" s="4">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="213" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A213" s="4">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="214" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A214" s="4">
+        <v>250</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
structy linked list challenges
</commit_message>
<xml_diff>
--- a/docs/Programming Puzzles.xlsx
+++ b/docs/Programming Puzzles.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\ProjectDSA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CE66EA5-BD36-4006-BAEE-AB8CA2FEE2E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6097609-F86C-4C71-BBBF-A491188BE6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1504" uniqueCount="537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1537" uniqueCount="550">
   <si>
     <t>PLATFORM</t>
   </si>
@@ -1650,6 +1650,45 @@
   </si>
   <si>
     <t>Just a variation of the one above.</t>
+  </si>
+  <si>
+    <t>Middle Value</t>
+  </si>
+  <si>
+    <t>18/10/2026</t>
+  </si>
+  <si>
+    <t>Solution uses the slow and fast pointer technique (also known as Floyd's two-pointer technique).</t>
+  </si>
+  <si>
+    <t>Can be solved with a set or with the slow/fast pointer technique.</t>
+  </si>
+  <si>
+    <t>Undupe Sorted Linked List</t>
+  </si>
+  <si>
+    <t>19/10/2026</t>
+  </si>
+  <si>
+    <t>Create Linked List</t>
+  </si>
+  <si>
+    <t>Build a Queue</t>
+  </si>
+  <si>
+    <t>Add Lists</t>
+  </si>
+  <si>
+    <t>Lowest Common Ancestor</t>
+  </si>
+  <si>
+    <t>Flip Tree</t>
+  </si>
+  <si>
+    <t>Login via X for AOC challenges.</t>
+  </si>
+  <si>
+    <t>https://adventofcode.com/2015/day/1</t>
   </si>
 </sst>
 </file>
@@ -2128,15 +2167,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E29EE35E-42CE-4BB8-BA9B-83E0DF36D658}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="53.42578125" customWidth="1"/>
+    <col min="1" max="1" width="53.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>422</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>548</v>
       </c>
     </row>
   </sheetData>
@@ -2146,9 +2190,50 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{673553DD-7322-43E4-B8E6-8596552AA633}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="33.90625" customWidth="1"/>
+    <col min="2" max="2" width="22.81640625" customWidth="1"/>
+    <col min="3" max="3" width="20.26953125" customWidth="1"/>
+    <col min="4" max="4" width="24.26953125" customWidth="1"/>
+    <col min="5" max="5" width="21.08984375" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="67" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>549</v>
+      </c>
+      <c r="E2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2156,21 +2241,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{758F6333-ADD2-4F62-82FC-3789A0207F8D}">
   <dimension ref="A1:J162"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" style="4" customWidth="1"/>
-    <col min="3" max="3" width="52.28515625" customWidth="1"/>
-    <col min="4" max="4" width="36.42578125" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" style="4" customWidth="1"/>
-    <col min="7" max="7" width="34.5703125" customWidth="1"/>
+    <col min="1" max="1" width="18.453125" customWidth="1"/>
+    <col min="2" max="2" width="11.81640625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="52.26953125" customWidth="1"/>
+    <col min="4" max="4" width="36.453125" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" customWidth="1"/>
+    <col min="6" max="6" width="13.54296875" style="4" customWidth="1"/>
+    <col min="7" max="7" width="34.54296875" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="15.28515625" customWidth="1"/>
-    <col min="10" max="10" width="92.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="15.26953125" customWidth="1"/>
+    <col min="10" max="10" width="92.7265625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2202,7 +2287,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2228,7 +2313,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2254,7 +2339,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>5</v>
       </c>
@@ -2284,7 +2369,7 @@
       </c>
       <c r="J4" s="9"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -2310,7 +2395,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -2339,7 +2424,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -2365,7 +2450,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -2394,7 +2479,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -2423,7 +2508,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -2452,7 +2537,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -2481,7 +2566,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -2510,7 +2595,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
         <v>5</v>
       </c>
@@ -2542,7 +2627,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>5</v>
       </c>
@@ -2568,7 +2653,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -2597,7 +2682,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>5</v>
       </c>
@@ -2623,7 +2708,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>5</v>
       </c>
@@ -2652,7 +2737,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>5</v>
       </c>
@@ -2681,7 +2766,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>5</v>
       </c>
@@ -2710,7 +2795,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>5</v>
       </c>
@@ -2739,7 +2824,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>5</v>
       </c>
@@ -2768,7 +2853,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
         <v>5</v>
       </c>
@@ -2800,7 +2885,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -2829,7 +2914,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>5</v>
       </c>
@@ -2858,7 +2943,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>5</v>
       </c>
@@ -2887,7 +2972,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>5</v>
       </c>
@@ -2913,7 +2998,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>5</v>
       </c>
@@ -2942,7 +3027,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>5</v>
       </c>
@@ -2971,7 +3056,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>5</v>
       </c>
@@ -3000,7 +3085,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>5</v>
       </c>
@@ -3029,7 +3114,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>5</v>
       </c>
@@ -3058,7 +3143,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>5</v>
       </c>
@@ -3087,7 +3172,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>5</v>
       </c>
@@ -3116,7 +3201,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>5</v>
       </c>
@@ -3145,7 +3230,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>5</v>
       </c>
@@ -3168,7 +3253,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>5</v>
       </c>
@@ -3191,7 +3276,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>5</v>
       </c>
@@ -3214,7 +3299,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>5</v>
       </c>
@@ -3243,7 +3328,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>5</v>
       </c>
@@ -3272,7 +3357,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>5</v>
       </c>
@@ -3301,7 +3386,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>5</v>
       </c>
@@ -3330,7 +3415,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>5</v>
       </c>
@@ -3356,7 +3441,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>5</v>
       </c>
@@ -3385,7 +3470,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>5</v>
       </c>
@@ -3414,7 +3499,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>5</v>
       </c>
@@ -3443,7 +3528,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>5</v>
       </c>
@@ -3469,7 +3554,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>5</v>
       </c>
@@ -3489,7 +3574,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>5</v>
       </c>
@@ -3509,7 +3594,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" s="7" t="s">
         <v>5</v>
       </c>
@@ -3539,7 +3624,7 @@
       </c>
       <c r="J49" s="9"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>5</v>
       </c>
@@ -3568,7 +3653,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>5</v>
       </c>
@@ -3597,7 +3682,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>5</v>
       </c>
@@ -3626,7 +3711,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>5</v>
       </c>
@@ -3655,7 +3740,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>5</v>
       </c>
@@ -3684,7 +3769,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>5</v>
       </c>
@@ -3713,7 +3798,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="56" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A56" s="10" t="s">
         <v>5</v>
       </c>
@@ -3745,7 +3830,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="57" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A57" s="10" t="s">
         <v>5</v>
       </c>
@@ -3775,7 +3860,7 @@
       </c>
       <c r="J57" s="12"/>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>5</v>
       </c>
@@ -3804,7 +3889,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>5</v>
       </c>
@@ -3830,7 +3915,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>5</v>
       </c>
@@ -3859,7 +3944,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>5</v>
       </c>
@@ -3888,7 +3973,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>5</v>
       </c>
@@ -3908,7 +3993,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>5</v>
       </c>
@@ -3928,7 +4013,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>5</v>
       </c>
@@ -3957,7 +4042,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>5</v>
       </c>
@@ -3986,7 +4071,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>5</v>
       </c>
@@ -4003,7 +4088,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>5</v>
       </c>
@@ -4032,7 +4117,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>5</v>
       </c>
@@ -4061,7 +4146,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="69" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A69" s="10" t="s">
         <v>5</v>
       </c>
@@ -4093,7 +4178,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="70" spans="1:10" s="7" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" s="7" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="7" t="s">
         <v>5</v>
       </c>
@@ -4125,7 +4210,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>5</v>
       </c>
@@ -4153,7 +4238,7 @@
       </c>
       <c r="J71"/>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>5</v>
       </c>
@@ -4182,7 +4267,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>5</v>
       </c>
@@ -4211,7 +4296,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="74" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A74" s="10" t="s">
         <v>5</v>
       </c>
@@ -4243,7 +4328,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>5</v>
       </c>
@@ -4266,7 +4351,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="76" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A76" s="10" t="s">
         <v>5</v>
       </c>
@@ -4298,7 +4383,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="77" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A77" s="10" t="s">
         <v>5</v>
       </c>
@@ -4330,7 +4415,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>5</v>
       </c>
@@ -4359,7 +4444,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>5</v>
       </c>
@@ -4388,7 +4473,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>5</v>
       </c>
@@ -4417,7 +4502,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>5</v>
       </c>
@@ -4443,7 +4528,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="82" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A82" s="10" t="s">
         <v>5</v>
       </c>
@@ -4475,7 +4560,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="83" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A83" s="10" t="s">
         <v>5</v>
       </c>
@@ -4505,7 +4590,7 @@
       </c>
       <c r="J83" s="12"/>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>5</v>
       </c>
@@ -4525,7 +4610,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="85" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A85" s="10" t="s">
         <v>5</v>
       </c>
@@ -4557,7 +4642,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>5</v>
       </c>
@@ -4586,7 +4671,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>5</v>
       </c>
@@ -4615,7 +4700,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>5</v>
       </c>
@@ -4644,7 +4729,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>5</v>
       </c>
@@ -4673,7 +4758,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>5</v>
       </c>
@@ -4699,7 +4784,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="91" spans="1:10" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" s="10" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A91" s="10" t="s">
         <v>5</v>
       </c>
@@ -4731,7 +4816,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="92" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A92" s="10" t="s">
         <v>5</v>
       </c>
@@ -4763,7 +4848,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>5</v>
       </c>
@@ -4792,7 +4877,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>5</v>
       </c>
@@ -4821,7 +4906,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>5</v>
       </c>
@@ -4850,7 +4935,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>321</v>
       </c>
@@ -4879,7 +4964,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="97" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A97" s="10" t="s">
         <v>5</v>
       </c>
@@ -4911,7 +4996,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>5</v>
       </c>
@@ -4931,7 +5016,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="99" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>5</v>
       </c>
@@ -4960,7 +5045,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>5</v>
       </c>
@@ -4989,7 +5074,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>5</v>
       </c>
@@ -5009,7 +5094,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>5</v>
       </c>
@@ -5032,7 +5117,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="103" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>5</v>
       </c>
@@ -5061,7 +5146,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="104" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A104" s="10" t="s">
         <v>5</v>
       </c>
@@ -5093,7 +5178,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="105" spans="1:10" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" s="10" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A105" s="10" t="s">
         <v>5</v>
       </c>
@@ -5125,7 +5210,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="106" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A106" s="10" t="s">
         <v>5</v>
       </c>
@@ -5157,7 +5242,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="107" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A107" s="10" t="s">
         <v>394</v>
       </c>
@@ -5189,7 +5274,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="108" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A108" s="10" t="s">
         <v>394</v>
       </c>
@@ -5221,7 +5306,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>5</v>
       </c>
@@ -5240,7 +5325,7 @@
       <c r="F109"/>
       <c r="J109"/>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>5</v>
       </c>
@@ -5269,7 +5354,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="111" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A111" s="10" t="s">
         <v>5</v>
       </c>
@@ -5301,7 +5386,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="112" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A112" s="10" t="s">
         <v>5</v>
       </c>
@@ -5333,7 +5418,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>5</v>
       </c>
@@ -5362,7 +5447,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>5</v>
       </c>
@@ -5391,7 +5476,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>5</v>
       </c>
@@ -5417,7 +5502,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="116" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A116" s="10" t="s">
         <v>5</v>
       </c>
@@ -5449,7 +5534,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="117" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A117" s="10" t="s">
         <v>5</v>
       </c>
@@ -5481,7 +5566,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>5</v>
       </c>
@@ -5510,7 +5595,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="119" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A119" s="10" t="s">
         <v>5</v>
       </c>
@@ -5542,7 +5627,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>5</v>
       </c>
@@ -5571,7 +5656,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>5</v>
       </c>
@@ -5597,7 +5682,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>5</v>
       </c>
@@ -5623,7 +5708,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>5</v>
       </c>
@@ -5649,7 +5734,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>5</v>
       </c>
@@ -5678,7 +5763,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>5</v>
       </c>
@@ -5707,7 +5792,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>5</v>
       </c>
@@ -5736,7 +5821,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="127" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A127" s="10" t="s">
         <v>5</v>
       </c>
@@ -5766,7 +5851,7 @@
       </c>
       <c r="J127" s="12"/>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>5</v>
       </c>
@@ -5795,7 +5880,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>5</v>
       </c>
@@ -5815,7 +5900,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>5</v>
       </c>
@@ -5835,7 +5920,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>5</v>
       </c>
@@ -5855,7 +5940,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>5</v>
       </c>
@@ -5875,7 +5960,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>5</v>
       </c>
@@ -5895,7 +5980,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>5</v>
       </c>
@@ -5921,7 +6006,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>5</v>
       </c>
@@ -5947,7 +6032,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>5</v>
       </c>
@@ -5976,7 +6061,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>5</v>
       </c>
@@ -6002,7 +6087,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>5</v>
       </c>
@@ -6031,7 +6116,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>5</v>
       </c>
@@ -6057,7 +6142,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>5</v>
       </c>
@@ -6083,7 +6168,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>5</v>
       </c>
@@ -6112,7 +6197,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>5</v>
       </c>
@@ -6138,7 +6223,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>5</v>
       </c>
@@ -6164,7 +6249,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>5</v>
       </c>
@@ -6190,7 +6275,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>321</v>
       </c>
@@ -6219,7 +6304,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A146" t="s">
         <v>321</v>
       </c>
@@ -6248,7 +6333,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>5</v>
       </c>
@@ -6268,7 +6353,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>5</v>
       </c>
@@ -6297,7 +6382,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>5</v>
       </c>
@@ -6326,7 +6411,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A150" t="s">
         <v>5</v>
       </c>
@@ -6355,7 +6440,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>5</v>
       </c>
@@ -6381,7 +6466,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>5</v>
       </c>
@@ -6407,7 +6492,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A153" t="s">
         <v>5</v>
       </c>
@@ -6436,7 +6521,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>5</v>
       </c>
@@ -6465,7 +6550,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A155" t="s">
         <v>5</v>
       </c>
@@ -6494,7 +6579,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>5</v>
       </c>
@@ -6523,7 +6608,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>5</v>
       </c>
@@ -6552,7 +6637,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>5</v>
       </c>
@@ -6581,7 +6666,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>5</v>
       </c>
@@ -6610,7 +6695,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>5</v>
       </c>
@@ -6639,7 +6724,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>5</v>
       </c>
@@ -6665,7 +6750,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A162" t="s">
         <v>5</v>
       </c>
@@ -6704,18 +6789,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63392036-0DF4-41BC-932A-0EBA4F02E5CB}">
   <dimension ref="A1:G211"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.7265625" customWidth="1"/>
     <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="3" max="3" width="23.85546875" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" customWidth="1"/>
-    <col min="7" max="7" width="111.140625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="23.81640625" customWidth="1"/>
+    <col min="4" max="4" width="14.1796875" customWidth="1"/>
+    <col min="5" max="5" width="15.26953125" customWidth="1"/>
+    <col min="6" max="6" width="14.7265625" customWidth="1"/>
+    <col min="7" max="7" width="111.1796875" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -6738,7 +6823,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
         <v>17</v>
       </c>
@@ -6758,7 +6843,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
         <v>18</v>
       </c>
@@ -6778,7 +6863,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <v>19</v>
       </c>
@@ -6788,7 +6873,7 @@
       <c r="E4" s="4"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>20</v>
       </c>
@@ -6798,7 +6883,7 @@
       <c r="E5" s="4"/>
       <c r="F5" s="13"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>21</v>
       </c>
@@ -6808,7 +6893,7 @@
       <c r="E6" s="4"/>
       <c r="F6" s="13"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>22</v>
       </c>
@@ -6818,7 +6903,7 @@
       <c r="E7" s="4"/>
       <c r="F7" s="13"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>23</v>
       </c>
@@ -6828,7 +6913,7 @@
       <c r="E8" s="4"/>
       <c r="F8" s="13"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>24</v>
       </c>
@@ -6838,7 +6923,7 @@
       <c r="E9" s="4"/>
       <c r="F9" s="13"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>25</v>
       </c>
@@ -6848,7 +6933,7 @@
       <c r="E10" s="4"/>
       <c r="F10" s="13"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>26</v>
       </c>
@@ -6858,7 +6943,7 @@
       <c r="E11" s="4"/>
       <c r="F11" s="13"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>27</v>
       </c>
@@ -6868,7 +6953,7 @@
       <c r="E12" s="4"/>
       <c r="F12" s="13"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>28</v>
       </c>
@@ -6878,7 +6963,7 @@
       <c r="E13" s="4"/>
       <c r="F13" s="13"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
         <v>29</v>
       </c>
@@ -6888,7 +6973,7 @@
       <c r="E14" s="4"/>
       <c r="F14" s="13"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
         <v>30</v>
       </c>
@@ -6898,7 +6983,7 @@
       <c r="E15" s="4"/>
       <c r="F15" s="13"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
         <v>31</v>
       </c>
@@ -6908,7 +6993,7 @@
       <c r="E16" s="4"/>
       <c r="F16" s="13"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
         <v>32</v>
       </c>
@@ -6918,7 +7003,7 @@
       <c r="E17" s="4"/>
       <c r="F17" s="13"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
         <v>33</v>
       </c>
@@ -6928,7 +7013,7 @@
       <c r="E18" s="4"/>
       <c r="F18" s="13"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
         <v>34</v>
       </c>
@@ -6938,7 +7023,7 @@
       <c r="E19" s="4"/>
       <c r="F19" s="13"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
         <v>35</v>
       </c>
@@ -6948,7 +7033,7 @@
       <c r="E20" s="4"/>
       <c r="F20" s="13"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="4">
         <v>36</v>
       </c>
@@ -6958,7 +7043,7 @@
       <c r="E21" s="4"/>
       <c r="F21" s="13"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="4">
         <v>37</v>
       </c>
@@ -6968,7 +7053,7 @@
       <c r="E22" s="4"/>
       <c r="F22" s="13"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="4">
         <v>38</v>
       </c>
@@ -6978,7 +7063,7 @@
       <c r="E23" s="4"/>
       <c r="F23" s="13"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="4">
         <v>39</v>
       </c>
@@ -6988,7 +7073,7 @@
       <c r="E24" s="4"/>
       <c r="F24" s="13"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="4">
         <v>40</v>
       </c>
@@ -6998,7 +7083,7 @@
       <c r="E25" s="4"/>
       <c r="F25" s="13"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="4">
         <v>41</v>
       </c>
@@ -7008,7 +7093,7 @@
       <c r="E26" s="4"/>
       <c r="F26" s="13"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="4">
         <v>42</v>
       </c>
@@ -7018,7 +7103,7 @@
       <c r="E27" s="4"/>
       <c r="F27" s="13"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="4">
         <v>43</v>
       </c>
@@ -7028,7 +7113,7 @@
       <c r="E28" s="4"/>
       <c r="F28" s="13"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="4">
         <v>44</v>
       </c>
@@ -7038,7 +7123,7 @@
       <c r="E29" s="4"/>
       <c r="F29" s="13"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="4">
         <v>45</v>
       </c>
@@ -7048,7 +7133,7 @@
       <c r="E30" s="4"/>
       <c r="F30" s="13"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="4">
         <v>46</v>
       </c>
@@ -7058,7 +7143,7 @@
       <c r="E31" s="4"/>
       <c r="F31" s="13"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="4">
         <v>47</v>
       </c>
@@ -7068,7 +7153,7 @@
       <c r="E32" s="4"/>
       <c r="F32" s="13"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="4">
         <v>48</v>
       </c>
@@ -7078,7 +7163,7 @@
       <c r="E33" s="4"/>
       <c r="F33" s="13"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="4">
         <v>49</v>
       </c>
@@ -7088,7 +7173,7 @@
       <c r="E34" s="4"/>
       <c r="F34" s="13"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="4">
         <v>50</v>
       </c>
@@ -7098,7 +7183,7 @@
       <c r="E35" s="4"/>
       <c r="F35" s="13"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="4">
         <v>51</v>
       </c>
@@ -7108,7 +7193,7 @@
       <c r="E36" s="4"/>
       <c r="F36" s="13"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="4">
         <v>52</v>
       </c>
@@ -7118,7 +7203,7 @@
       <c r="E37" s="4"/>
       <c r="F37" s="13"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" s="4">
         <v>53</v>
       </c>
@@ -7128,7 +7213,7 @@
       <c r="E38" s="4"/>
       <c r="F38" s="13"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" s="4">
         <v>54</v>
       </c>
@@ -7138,7 +7223,7 @@
       <c r="E39" s="4"/>
       <c r="F39" s="13"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" s="4">
         <v>55</v>
       </c>
@@ -7148,7 +7233,7 @@
       <c r="E40" s="4"/>
       <c r="F40" s="13"/>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" s="4">
         <v>56</v>
       </c>
@@ -7158,7 +7243,7 @@
       <c r="E41" s="4"/>
       <c r="F41" s="13"/>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" s="4">
         <v>57</v>
       </c>
@@ -7168,7 +7253,7 @@
       <c r="E42" s="4"/>
       <c r="F42" s="13"/>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" s="4">
         <v>58</v>
       </c>
@@ -7178,7 +7263,7 @@
       <c r="E43" s="4"/>
       <c r="F43" s="13"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" s="4">
         <v>59</v>
       </c>
@@ -7188,7 +7273,7 @@
       <c r="E44" s="4"/>
       <c r="F44" s="13"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" s="4">
         <v>60</v>
       </c>
@@ -7198,7 +7283,7 @@
       <c r="E45" s="4"/>
       <c r="F45" s="13"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" s="4">
         <v>61</v>
       </c>
@@ -7208,7 +7293,7 @@
       <c r="E46" s="4"/>
       <c r="F46" s="13"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" s="4">
         <v>62</v>
       </c>
@@ -7218,7 +7303,7 @@
       <c r="E47" s="4"/>
       <c r="F47" s="13"/>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" s="4">
         <v>63</v>
       </c>
@@ -7228,7 +7313,7 @@
       <c r="E48" s="4"/>
       <c r="F48" s="13"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" s="4">
         <v>64</v>
       </c>
@@ -7238,7 +7323,7 @@
       <c r="E49" s="4"/>
       <c r="F49" s="13"/>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="4">
         <v>65</v>
       </c>
@@ -7248,7 +7333,7 @@
       <c r="E50" s="4"/>
       <c r="F50" s="13"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" s="4">
         <v>66</v>
       </c>
@@ -7258,7 +7343,7 @@
       <c r="E51" s="4"/>
       <c r="F51" s="13"/>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" s="4">
         <v>67</v>
       </c>
@@ -7268,7 +7353,7 @@
       <c r="E52" s="4"/>
       <c r="F52" s="13"/>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" s="4">
         <v>68</v>
       </c>
@@ -7278,7 +7363,7 @@
       <c r="E53" s="4"/>
       <c r="F53" s="13"/>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" s="4">
         <v>69</v>
       </c>
@@ -7288,7 +7373,7 @@
       <c r="E54" s="4"/>
       <c r="F54" s="13"/>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" s="4">
         <v>70</v>
       </c>
@@ -7298,7 +7383,7 @@
       <c r="E55" s="4"/>
       <c r="F55" s="13"/>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="4">
         <v>71</v>
       </c>
@@ -7308,7 +7393,7 @@
       <c r="E56" s="4"/>
       <c r="F56" s="13"/>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" s="4">
         <v>72</v>
       </c>
@@ -7318,7 +7403,7 @@
       <c r="E57" s="4"/>
       <c r="F57" s="13"/>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" s="4">
         <v>73</v>
       </c>
@@ -7328,7 +7413,7 @@
       <c r="E58" s="4"/>
       <c r="F58" s="13"/>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" s="4">
         <v>74</v>
       </c>
@@ -7338,7 +7423,7 @@
       <c r="E59" s="4"/>
       <c r="F59" s="13"/>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" s="4">
         <v>75</v>
       </c>
@@ -7348,7 +7433,7 @@
       <c r="E60" s="4"/>
       <c r="F60" s="13"/>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="4">
         <v>76</v>
       </c>
@@ -7358,7 +7443,7 @@
       <c r="E61" s="4"/>
       <c r="F61" s="13"/>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" s="4">
         <v>77</v>
       </c>
@@ -7368,7 +7453,7 @@
       <c r="E62" s="4"/>
       <c r="F62" s="13"/>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" s="4">
         <v>78</v>
       </c>
@@ -7378,7 +7463,7 @@
       <c r="E63" s="4"/>
       <c r="F63" s="13"/>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" s="4">
         <v>79</v>
       </c>
@@ -7388,7 +7473,7 @@
       <c r="E64" s="4"/>
       <c r="F64" s="13"/>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" s="4">
         <v>80</v>
       </c>
@@ -7398,7 +7483,7 @@
       <c r="E65" s="4"/>
       <c r="F65" s="13"/>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" s="4">
         <v>81</v>
       </c>
@@ -7408,7 +7493,7 @@
       <c r="E66" s="4"/>
       <c r="F66" s="13"/>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" s="4">
         <v>82</v>
       </c>
@@ -7418,7 +7503,7 @@
       <c r="E67" s="4"/>
       <c r="F67" s="13"/>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" s="4">
         <v>83</v>
       </c>
@@ -7428,7 +7513,7 @@
       <c r="E68" s="4"/>
       <c r="F68" s="13"/>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" s="4">
         <v>84</v>
       </c>
@@ -7438,7 +7523,7 @@
       <c r="E69" s="4"/>
       <c r="F69" s="13"/>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="4">
         <v>85</v>
       </c>
@@ -7448,7 +7533,7 @@
       <c r="E70" s="4"/>
       <c r="F70" s="13"/>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" s="4">
         <v>86</v>
       </c>
@@ -7458,7 +7543,7 @@
       <c r="E71" s="4"/>
       <c r="F71" s="13"/>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" s="4">
         <v>87</v>
       </c>
@@ -7468,7 +7553,7 @@
       <c r="E72" s="4"/>
       <c r="F72" s="13"/>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" s="4">
         <v>88</v>
       </c>
@@ -7478,7 +7563,7 @@
       <c r="E73" s="4"/>
       <c r="F73" s="13"/>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" s="4">
         <v>89</v>
       </c>
@@ -7488,7 +7573,7 @@
       <c r="E74" s="4"/>
       <c r="F74" s="13"/>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" s="4">
         <v>90</v>
       </c>
@@ -7498,7 +7583,7 @@
       <c r="E75" s="4"/>
       <c r="F75" s="13"/>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" s="4">
         <v>91</v>
       </c>
@@ -7508,7 +7593,7 @@
       <c r="E76" s="4"/>
       <c r="F76" s="13"/>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" s="4">
         <v>92</v>
       </c>
@@ -7518,7 +7603,7 @@
       <c r="E77" s="4"/>
       <c r="F77" s="13"/>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" s="4">
         <v>93</v>
       </c>
@@ -7528,7 +7613,7 @@
       <c r="E78" s="4"/>
       <c r="F78" s="13"/>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" s="4">
         <v>94</v>
       </c>
@@ -7538,7 +7623,7 @@
       <c r="E79" s="4"/>
       <c r="F79" s="13"/>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="4">
         <v>95</v>
       </c>
@@ -7556,7 +7641,7 @@
       </c>
       <c r="F80" s="13"/>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A81" s="4">
         <v>99</v>
       </c>
@@ -7577,7 +7662,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A82" s="4">
         <v>100</v>
       </c>
@@ -7598,7 +7683,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A83" s="4">
         <v>103</v>
       </c>
@@ -7619,7 +7704,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A84" s="4">
         <v>104</v>
       </c>
@@ -7640,7 +7725,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A85" s="4">
         <v>105</v>
       </c>
@@ -7661,7 +7746,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A86" s="4">
         <v>106</v>
       </c>
@@ -7682,7 +7767,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A87" s="4">
         <v>107</v>
       </c>
@@ -7703,7 +7788,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A88" s="4">
         <v>109</v>
       </c>
@@ -7726,7 +7811,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" s="4">
         <v>110</v>
       </c>
@@ -7749,7 +7834,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A90" s="4">
         <v>111</v>
       </c>
@@ -7772,7 +7857,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A91" s="4">
         <v>112</v>
       </c>
@@ -7795,7 +7880,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A92" s="4">
         <v>113</v>
       </c>
@@ -7818,7 +7903,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A93" s="4">
         <v>114</v>
       </c>
@@ -7841,7 +7926,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A94" s="4">
         <v>117</v>
       </c>
@@ -7861,7 +7946,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A95" s="4">
         <v>118</v>
       </c>
@@ -7881,7 +7966,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A96" s="4">
         <v>119</v>
       </c>
@@ -7904,7 +7989,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97" s="4">
         <v>120</v>
       </c>
@@ -7927,7 +8012,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98" s="4">
         <v>121</v>
       </c>
@@ -7947,7 +8032,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" s="4">
         <v>124</v>
       </c>
@@ -7967,7 +8052,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" s="4">
         <v>125</v>
       </c>
@@ -7990,7 +8075,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" s="4">
         <v>126</v>
       </c>
@@ -8013,7 +8098,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" s="4">
         <v>128</v>
       </c>
@@ -8033,7 +8118,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103" s="4">
         <v>129</v>
       </c>
@@ -8056,7 +8141,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104" s="4">
         <v>130</v>
       </c>
@@ -8079,7 +8164,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" s="4">
         <v>131</v>
       </c>
@@ -8102,7 +8187,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="106" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A106" s="14">
         <v>132</v>
       </c>
@@ -8125,7 +8210,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" s="4">
         <v>133</v>
       </c>
@@ -8148,7 +8233,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" s="4">
         <v>137</v>
       </c>
@@ -8171,7 +8256,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" s="4">
         <v>138</v>
       </c>
@@ -8191,7 +8276,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" s="4">
         <v>139</v>
       </c>
@@ -8214,7 +8299,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" s="4">
         <v>140</v>
       </c>
@@ -8237,7 +8322,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="112" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" s="4">
         <v>141</v>
       </c>
@@ -8260,7 +8345,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A113" s="4">
         <v>143</v>
       </c>
@@ -8283,7 +8368,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A114" s="4">
         <v>144</v>
       </c>
@@ -8303,7 +8388,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A115" s="4">
         <v>145</v>
       </c>
@@ -8326,7 +8411,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="116" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A116" s="14">
         <v>146</v>
       </c>
@@ -8349,7 +8434,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A117" s="4">
         <v>147</v>
       </c>
@@ -8369,7 +8454,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="118" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A118" s="4">
         <v>149</v>
       </c>
@@ -8392,7 +8477,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A119" s="4">
         <v>150</v>
       </c>
@@ -8415,7 +8500,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A120" s="4">
         <v>151</v>
       </c>
@@ -8435,7 +8520,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A121" s="4">
         <v>152</v>
       </c>
@@ -8458,7 +8543,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A122" s="4">
         <v>153</v>
       </c>
@@ -8478,7 +8563,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A123" s="4">
         <v>154</v>
       </c>
@@ -8498,7 +8583,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="124" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A124" s="14">
         <v>155</v>
       </c>
@@ -8519,7 +8604,7 @@
       </c>
       <c r="G124" s="19"/>
     </row>
-    <row r="125" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A125" s="14">
         <v>156</v>
       </c>
@@ -8542,7 +8627,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A126" s="4">
         <v>160</v>
       </c>
@@ -8562,7 +8647,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A127" s="4">
         <v>161</v>
       </c>
@@ -8585,7 +8670,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="128" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A128" s="4">
         <v>162</v>
       </c>
@@ -8608,7 +8693,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A129" s="4">
         <v>163</v>
       </c>
@@ -8631,7 +8716,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A130" s="4">
         <v>164</v>
       </c>
@@ -8654,7 +8739,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A131" s="4">
         <v>167</v>
       </c>
@@ -8677,7 +8762,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A132" s="4">
         <v>168</v>
       </c>
@@ -8700,7 +8785,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="133" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A133" s="14">
         <v>169</v>
       </c>
@@ -8723,7 +8808,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A134" s="4">
         <v>171</v>
       </c>
@@ -8746,7 +8831,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A135" s="4">
         <v>172</v>
       </c>
@@ -8769,7 +8854,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A136" s="4">
         <v>174</v>
       </c>
@@ -8792,7 +8877,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A137" s="4">
         <v>175</v>
       </c>
@@ -8815,7 +8900,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A138" s="4">
         <v>177</v>
       </c>
@@ -8825,105 +8910,159 @@
       <c r="C138" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="D138" s="4"/>
+      <c r="D138" s="4">
+        <v>1</v>
+      </c>
       <c r="E138" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="F138" s="4"/>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F138" s="4" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A139" s="4">
         <v>178</v>
       </c>
-      <c r="B139" s="4"/>
+      <c r="B139" s="4" t="s">
+        <v>537</v>
+      </c>
       <c r="C139" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="D139" s="4"/>
-      <c r="E139" s="4"/>
-      <c r="F139" s="4"/>
-    </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D139" s="4">
+        <v>1</v>
+      </c>
+      <c r="E139" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F139" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="G139" s="5" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A140" s="4">
         <v>179</v>
       </c>
-      <c r="B140" s="4"/>
+      <c r="B140" s="4" t="s">
+        <v>116</v>
+      </c>
       <c r="C140" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="D140" s="4"/>
-      <c r="E140" s="4"/>
-      <c r="F140" s="4"/>
-    </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D140" s="4">
+        <v>1</v>
+      </c>
+      <c r="E140" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F140" s="4" t="s">
+        <v>538</v>
+      </c>
+      <c r="G140" s="5" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A141" s="4">
         <v>180</v>
       </c>
-      <c r="B141" s="4"/>
+      <c r="B141" s="4" t="s">
+        <v>541</v>
+      </c>
       <c r="C141" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D141" s="4"/>
-      <c r="E141" s="4"/>
-      <c r="F141" s="4"/>
-    </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E141" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F141" s="4" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A142" s="4">
         <v>181</v>
       </c>
-      <c r="B142" s="4"/>
+      <c r="B142" s="4" t="s">
+        <v>543</v>
+      </c>
       <c r="C142" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D142" s="4"/>
-      <c r="E142" s="4"/>
-      <c r="F142" s="4"/>
-    </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E142" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F142" s="4" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A143" s="4">
         <v>182</v>
       </c>
-      <c r="B143" s="4"/>
+      <c r="B143" s="4" t="s">
+        <v>544</v>
+      </c>
       <c r="C143" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D143" s="4"/>
-      <c r="E143" s="4"/>
+      <c r="E143" s="4" t="s">
+        <v>366</v>
+      </c>
       <c r="F143" s="4"/>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A144" s="4">
         <v>183</v>
       </c>
-      <c r="B144" s="4"/>
+      <c r="B144" s="4" t="s">
+        <v>545</v>
+      </c>
       <c r="C144" s="4" t="s">
         <v>112</v>
       </c>
       <c r="D144" s="4"/>
-      <c r="E144" s="4"/>
+      <c r="E144" s="4" t="s">
+        <v>366</v>
+      </c>
       <c r="F144" s="4"/>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A145" s="4">
         <v>184</v>
       </c>
-      <c r="B145" s="4"/>
-      <c r="C145" s="4"/>
+      <c r="B145" s="4" t="s">
+        <v>546</v>
+      </c>
+      <c r="C145" s="4" t="s">
+        <v>126</v>
+      </c>
       <c r="D145" s="4"/>
       <c r="E145" s="4"/>
       <c r="F145" s="4"/>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A146" s="4">
         <v>185</v>
       </c>
-      <c r="B146" s="4"/>
-      <c r="C146" s="4"/>
+      <c r="B146" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="C146" s="4" t="s">
+        <v>126</v>
+      </c>
       <c r="D146" s="4"/>
       <c r="E146" s="4"/>
       <c r="F146" s="4"/>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A147" s="4">
         <v>186</v>
       </c>
@@ -8933,7 +9072,7 @@
       <c r="E147" s="4"/>
       <c r="F147" s="4"/>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A148" s="4">
         <v>187</v>
       </c>
@@ -8943,7 +9082,7 @@
       <c r="E148" s="4"/>
       <c r="F148" s="4"/>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A149" s="4">
         <v>188</v>
       </c>
@@ -8953,7 +9092,7 @@
       <c r="E149" s="4"/>
       <c r="F149" s="4"/>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A150" s="4">
         <v>189</v>
       </c>
@@ -8963,7 +9102,7 @@
       <c r="E150" s="4"/>
       <c r="F150" s="4"/>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A151" s="4">
         <v>190</v>
       </c>
@@ -8973,7 +9112,7 @@
       <c r="E151" s="4"/>
       <c r="F151" s="4"/>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A152" s="4">
         <v>191</v>
       </c>
@@ -8983,7 +9122,7 @@
       <c r="E152" s="4"/>
       <c r="F152" s="4"/>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A153" s="4">
         <v>192</v>
       </c>
@@ -8993,7 +9132,7 @@
       <c r="E153" s="4"/>
       <c r="F153" s="4"/>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A154" s="4">
         <v>193</v>
       </c>
@@ -9003,7 +9142,7 @@
       <c r="E154" s="4"/>
       <c r="F154" s="4"/>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A155" s="4">
         <v>194</v>
       </c>
@@ -9013,7 +9152,7 @@
       <c r="E155" s="4"/>
       <c r="F155" s="4"/>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A156" s="4">
         <v>195</v>
       </c>
@@ -9023,7 +9162,7 @@
       <c r="E156" s="4"/>
       <c r="F156" s="4"/>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A157" s="4">
         <v>196</v>
       </c>
@@ -9033,7 +9172,7 @@
       <c r="E157" s="4"/>
       <c r="F157" s="4"/>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A158" s="4">
         <v>197</v>
       </c>
@@ -9043,7 +9182,7 @@
       <c r="E158" s="4"/>
       <c r="F158" s="4"/>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A159" s="4">
         <v>198</v>
       </c>
@@ -9053,7 +9192,7 @@
       <c r="E159" s="4"/>
       <c r="F159" s="4"/>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A160" s="4">
         <v>199</v>
       </c>
@@ -9063,7 +9202,7 @@
       <c r="E160" s="4"/>
       <c r="F160" s="4"/>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A161" s="4">
         <v>200</v>
       </c>
@@ -9073,7 +9212,7 @@
       <c r="E161" s="4"/>
       <c r="F161" s="4"/>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A162" s="4">
         <v>201</v>
       </c>
@@ -9083,7 +9222,7 @@
       <c r="E162" s="4"/>
       <c r="F162" s="4"/>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A163" s="4">
         <v>202</v>
       </c>
@@ -9093,7 +9232,7 @@
       <c r="E163" s="4"/>
       <c r="F163" s="4"/>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A164" s="4">
         <v>203</v>
       </c>
@@ -9103,235 +9242,235 @@
       <c r="E164" s="4"/>
       <c r="F164" s="4"/>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A165" s="4">
         <v>204</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A166" s="4">
         <v>205</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A167" s="4">
         <v>206</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A168" s="4">
         <v>207</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A169" s="4">
         <v>208</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A170" s="4">
         <v>209</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A171" s="4">
         <v>210</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A172" s="4">
         <v>211</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A173" s="4">
         <v>212</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A174" s="4">
         <v>213</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A175" s="4">
         <v>214</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A176" s="4">
         <v>215</v>
       </c>
     </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A177" s="4">
         <v>216</v>
       </c>
     </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A178" s="4">
         <v>217</v>
       </c>
     </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A179" s="4">
         <v>218</v>
       </c>
     </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A180" s="4">
         <v>219</v>
       </c>
     </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A181" s="4">
         <v>220</v>
       </c>
     </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A182" s="4">
         <v>221</v>
       </c>
     </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A183" s="4">
         <v>222</v>
       </c>
     </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A184" s="4">
         <v>223</v>
       </c>
     </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A185" s="4">
         <v>224</v>
       </c>
     </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A186" s="4">
         <v>225</v>
       </c>
     </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A187" s="4">
         <v>226</v>
       </c>
     </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A188" s="4">
         <v>227</v>
       </c>
     </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A189" s="4">
         <v>228</v>
       </c>
     </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A190" s="4">
         <v>229</v>
       </c>
     </row>
-    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A191" s="4">
         <v>230</v>
       </c>
     </row>
-    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A192" s="4">
         <v>231</v>
       </c>
     </row>
-    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A193" s="4">
         <v>232</v>
       </c>
     </row>
-    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A194" s="4">
         <v>233</v>
       </c>
     </row>
-    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A195" s="4">
         <v>234</v>
       </c>
     </row>
-    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A196" s="4">
         <v>235</v>
       </c>
     </row>
-    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A197" s="4">
         <v>236</v>
       </c>
     </row>
-    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A198" s="4">
         <v>237</v>
       </c>
     </row>
-    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A199" s="4">
         <v>238</v>
       </c>
     </row>
-    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A200" s="4">
         <v>239</v>
       </c>
     </row>
-    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A201" s="4">
         <v>240</v>
       </c>
     </row>
-    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A202" s="4">
         <v>241</v>
       </c>
     </row>
-    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A203" s="4">
         <v>242</v>
       </c>
     </row>
-    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A204" s="4">
         <v>243</v>
       </c>
     </row>
-    <row r="205" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A205" s="4">
         <v>244</v>
       </c>
     </row>
-    <row r="206" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A206" s="4">
         <v>245</v>
       </c>
     </row>
-    <row r="207" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A207" s="4">
         <v>246</v>
       </c>
     </row>
-    <row r="208" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A208" s="4">
         <v>247</v>
       </c>
     </row>
-    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A209" s="4">
         <v>248</v>
       </c>
     </row>
-    <row r="210" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A210" s="4"/>
     </row>
-    <row r="211" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A211" s="4"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
structy binary tree challenges
</commit_message>
<xml_diff>
--- a/docs/Programming Puzzles.xlsx
+++ b/docs/Programming Puzzles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\ProjectDSA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CABFCA72-0B05-4A3F-BDDE-B930545130D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E79CB979-5E9D-4B6B-8D43-7F762843BCD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1864" uniqueCount="555">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1566" uniqueCount="564">
   <si>
     <t>PLATFORM</t>
   </si>
@@ -1704,6 +1704,33 @@
   </si>
   <si>
     <t>Use dummy empty node pattern for iterative solution. Recursive solution is elegant.</t>
+  </si>
+  <si>
+    <t>21/10/2026</t>
+  </si>
+  <si>
+    <t>Trick: Get paths to the two nodes and then find the first common value among the paths. Use the Path Finder algorithm to find the intersection.</t>
+  </si>
+  <si>
+    <t>Lefty Nodes</t>
+  </si>
+  <si>
+    <t>Classic binary tree problem. Also known as the Invert Binary Tree problem, only difference is we're doing this in place instead of creating any Nodes.</t>
+  </si>
+  <si>
+    <t>Tricky part is coming up with the strategy. Base case with the length of the array matching the level is the main trick.</t>
+  </si>
+  <si>
+    <t>Binary Search Tree Includes</t>
+  </si>
+  <si>
+    <t>Is Binary Search Tree</t>
+  </si>
+  <si>
+    <t>Inorder traversal followed by sorted list check if it's in order.</t>
+  </si>
+  <si>
+    <t>Post Order</t>
   </si>
 </sst>
 </file>
@@ -9073,7 +9100,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A145" s="4">
         <v>184</v>
       </c>
@@ -9083,11 +9110,20 @@
       <c r="C145" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="D145" s="4"/>
-      <c r="E145" s="4"/>
-      <c r="F145" s="4"/>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D145" s="4">
+        <v>2</v>
+      </c>
+      <c r="E145" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F145" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="G145" s="5" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A146" s="4">
         <v>185</v>
       </c>
@@ -9097,51 +9133,102 @@
       <c r="C146" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="D146" s="4"/>
-      <c r="E146" s="4"/>
-      <c r="F146" s="4"/>
-    </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D146" s="4">
+        <v>2</v>
+      </c>
+      <c r="E146" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F146" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="G146" s="5" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A147" s="4">
         <v>186</v>
       </c>
-      <c r="B147" s="4"/>
-      <c r="C147" s="4"/>
-      <c r="D147" s="4"/>
-      <c r="E147" s="4"/>
-      <c r="F147" s="4"/>
-    </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B147" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="C147" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D147" s="4">
+        <v>3</v>
+      </c>
+      <c r="E147" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F147" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="G147" s="5" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A148" s="4">
         <v>187</v>
       </c>
-      <c r="B148" s="4"/>
-      <c r="C148" s="4"/>
-      <c r="D148" s="4"/>
-      <c r="E148" s="4"/>
-      <c r="F148" s="4"/>
-    </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B148" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="C148" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D148" s="4">
+        <v>1</v>
+      </c>
+      <c r="E148" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F148" s="4" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A149" s="4">
         <v>188</v>
       </c>
-      <c r="B149" s="4"/>
-      <c r="C149" s="4"/>
-      <c r="D149" s="4"/>
-      <c r="E149" s="4"/>
-      <c r="F149" s="4"/>
-    </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B149" s="4" t="s">
+        <v>561</v>
+      </c>
+      <c r="C149" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D149" s="4">
+        <v>2</v>
+      </c>
+      <c r="E149" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F149" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="G149" s="5" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A150" s="4">
         <v>189</v>
       </c>
-      <c r="B150" s="4"/>
-      <c r="C150" s="4"/>
+      <c r="B150" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="C150" s="4" t="s">
+        <v>126</v>
+      </c>
       <c r="D150" s="4"/>
-      <c r="E150" s="4"/>
+      <c r="E150" s="4" t="s">
+        <v>366</v>
+      </c>
       <c r="F150" s="4"/>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A151" s="4">
         <v>190</v>
       </c>
@@ -9151,7 +9238,7 @@
       <c r="E151" s="4"/>
       <c r="F151" s="4"/>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A152" s="4">
         <v>191</v>
       </c>
@@ -9161,7 +9248,7 @@
       <c r="E152" s="4"/>
       <c r="F152" s="4"/>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A153" s="4">
         <v>192</v>
       </c>
@@ -9171,7 +9258,7 @@
       <c r="E153" s="4"/>
       <c r="F153" s="4"/>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A154" s="4">
         <v>193</v>
       </c>
@@ -9181,7 +9268,7 @@
       <c r="E154" s="4"/>
       <c r="F154" s="4"/>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A155" s="4">
         <v>194</v>
       </c>
@@ -9191,7 +9278,7 @@
       <c r="E155" s="4"/>
       <c r="F155" s="4"/>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A156" s="4">
         <v>195</v>
       </c>
@@ -9201,7 +9288,7 @@
       <c r="E156" s="4"/>
       <c r="F156" s="4"/>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A157" s="4">
         <v>196</v>
       </c>
@@ -9211,7 +9298,7 @@
       <c r="E157" s="4"/>
       <c r="F157" s="4"/>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A158" s="4">
         <v>197</v>
       </c>
@@ -9221,7 +9308,7 @@
       <c r="E158" s="4"/>
       <c r="F158" s="4"/>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A159" s="4">
         <v>198</v>
       </c>
@@ -9231,7 +9318,7 @@
       <c r="E159" s="4"/>
       <c r="F159" s="4"/>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A160" s="4">
         <v>199</v>
       </c>

</xml_diff>

<commit_message>
structy exhaustive recursion challenges
</commit_message>
<xml_diff>
--- a/docs/Programming Puzzles.xlsx
+++ b/docs/Programming Puzzles.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\ProjectDSA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2781976-39B5-4BBC-9BC8-7B22D40F9D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34060D94-DD56-4CE0-8832-3E6E2FE06CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1626" uniqueCount="587">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1635" uniqueCount="591">
   <si>
     <t>PLATFORM</t>
   </si>
@@ -1800,6 +1800,18 @@
   </si>
   <si>
     <t>Substitute Synonyms</t>
+  </si>
+  <si>
+    <t>This takes some getting used to.</t>
+  </si>
+  <si>
+    <t>Order doesn't matter so lets solve with the subsets pattern.</t>
+  </si>
+  <si>
+    <t>Part One</t>
+  </si>
+  <si>
+    <t>Part Two</t>
   </si>
 </sst>
 </file>
@@ -2301,7 +2313,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{673553DD-7322-43E4-B8E6-8596552AA633}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.85546875" customWidth="1"/>
@@ -2340,7 +2352,21 @@
       <c r="A2" t="s">
         <v>549</v>
       </c>
+      <c r="B2" t="s">
+        <v>589</v>
+      </c>
       <c r="E2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>549</v>
+      </c>
+      <c r="B3" t="s">
+        <v>590</v>
+      </c>
+      <c r="E3" t="s">
         <v>366</v>
       </c>
     </row>
@@ -9469,11 +9495,17 @@
       <c r="C158" s="4" t="s">
         <v>580</v>
       </c>
+      <c r="D158" s="4">
+        <v>3</v>
+      </c>
       <c r="E158" s="4" t="s">
         <v>366</v>
       </c>
       <c r="F158" s="4" t="s">
         <v>576</v>
+      </c>
+      <c r="G158" s="5" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.25">
@@ -9486,22 +9518,40 @@
       <c r="C159" s="4" t="s">
         <v>580</v>
       </c>
+      <c r="D159" s="4">
+        <v>3</v>
+      </c>
       <c r="E159" s="4" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A160" s="4">
+      <c r="F159" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="G159" s="5" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="14">
         <v>208</v>
       </c>
-      <c r="B160" s="4" t="s">
+      <c r="B160" s="14" t="s">
         <v>581</v>
       </c>
-      <c r="C160" s="4" t="s">
+      <c r="C160" s="14" t="s">
         <v>580</v>
       </c>
-      <c r="E160" s="4" t="s">
-        <v>366</v>
+      <c r="D160" s="14">
+        <v>4</v>
+      </c>
+      <c r="E160" s="14" t="s">
+        <v>366</v>
+      </c>
+      <c r="F160" s="14" t="s">
+        <v>576</v>
+      </c>
+      <c r="G160" s="19" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
structy and aoc challenges
</commit_message>
<xml_diff>
--- a/docs/Programming Puzzles.xlsx
+++ b/docs/Programming Puzzles.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\ProjectDSA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34060D94-DD56-4CE0-8832-3E6E2FE06CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6B67631-3BC3-4E09-A70F-51395E3ABFA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1635" uniqueCount="591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1639" uniqueCount="595">
   <si>
     <t>PLATFORM</t>
   </si>
@@ -1812,6 +1812,18 @@
   </si>
   <si>
     <t>Part Two</t>
+  </si>
+  <si>
+    <t>25/10/2026</t>
+  </si>
+  <si>
+    <t>Subsets pattern. Tough one!</t>
+  </si>
+  <si>
+    <t>26/10/2026</t>
+  </si>
+  <si>
+    <t>Permutations pattern since order matters. Patterns are starting to make a little more sense...</t>
   </si>
 </sst>
 </file>
@@ -9554,7 +9566,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A161" s="4">
         <v>209</v>
       </c>
@@ -9564,11 +9576,20 @@
       <c r="C161" s="4" t="s">
         <v>580</v>
       </c>
+      <c r="D161" s="4">
+        <v>4</v>
+      </c>
       <c r="E161" s="4" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F161" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="G161" s="5" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A162" s="4">
         <v>210</v>
       </c>
@@ -9578,11 +9599,20 @@
       <c r="C162" s="4" t="s">
         <v>580</v>
       </c>
+      <c r="D162" s="4">
+        <v>4</v>
+      </c>
       <c r="E162" s="4" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F162" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="G162" s="5" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A163" s="4">
         <v>211</v>
       </c>
@@ -9596,7 +9626,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A164" s="4">
         <v>212</v>
       </c>
@@ -9610,7 +9640,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A165" s="4">
         <v>213</v>
       </c>
@@ -9624,57 +9654,57 @@
         <v>366</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" s="4">
         <v>214</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" s="4">
         <v>215</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" s="4">
         <v>216</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" s="4">
         <v>217</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" s="4">
         <v>218</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" s="4">
         <v>219</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" s="4">
         <v>220</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" s="4">
         <v>221</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" s="4">
         <v>222</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" s="4">
         <v>223</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176" s="4">
         <v>224</v>
       </c>

</xml_diff>

<commit_message>
aoc and structy challenges
</commit_message>
<xml_diff>
--- a/docs/Programming Puzzles.xlsx
+++ b/docs/Programming Puzzles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\ProjectDSA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6B67631-3BC3-4E09-A70F-51395E3ABFA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2372690-C255-4A30-9D9E-07ECAB16969A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1639" uniqueCount="595">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1686" uniqueCount="600">
   <si>
     <t>PLATFORM</t>
   </si>
@@ -1824,6 +1824,21 @@
   </si>
   <si>
     <t>Permutations pattern since order matters. Patterns are starting to make a little more sense...</t>
+  </si>
+  <si>
+    <t>https://adventofcode.com/2015/day/2</t>
+  </si>
+  <si>
+    <t>https://adventofcode.com/2015/day/3</t>
+  </si>
+  <si>
+    <t>Topological Order is to visit parents before children.</t>
+  </si>
+  <si>
+    <t>27/10/2026</t>
+  </si>
+  <si>
+    <t>Beautiful Code!</t>
   </si>
 </sst>
 </file>
@@ -1914,7 +1929,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1965,6 +1980,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Good" xfId="2" builtinId="26"/>
@@ -2325,13 +2341,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{673553DD-7322-43E4-B8E6-8596552AA633}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.85546875" customWidth="1"/>
+    <col min="1" max="1" width="37" customWidth="1"/>
     <col min="2" max="2" width="22.85546875" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" style="4" customWidth="1"/>
     <col min="5" max="5" width="21.140625" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="67" customWidth="1"/>
@@ -2347,7 +2363,7 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>367</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -2361,28 +2377,242 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="20" t="s">
         <v>549</v>
       </c>
       <c r="B2" t="s">
         <v>589</v>
       </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="4">
+        <v>1</v>
+      </c>
       <c r="E2" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="20" t="s">
         <v>549</v>
       </c>
       <c r="B3" t="s">
         <v>590</v>
       </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="4">
+        <v>1</v>
+      </c>
       <c r="E3" t="s">
         <v>366</v>
       </c>
     </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="20" t="s">
+        <v>595</v>
+      </c>
+      <c r="B4" t="s">
+        <v>589</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="20" t="s">
+        <v>595</v>
+      </c>
+      <c r="B5" t="s">
+        <v>590</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="4">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="20" t="s">
+        <v>596</v>
+      </c>
+      <c r="B6" t="s">
+        <v>589</v>
+      </c>
+      <c r="C6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="20" t="s">
+        <v>596</v>
+      </c>
+      <c r="B7" t="s">
+        <v>590</v>
+      </c>
+      <c r="C7" t="s">
+        <v>183</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E9" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E11" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E14" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E15" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E16" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E17" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="18" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E18" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E19" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E20" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E21" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="22" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E22" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="23" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E23" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E24" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="25" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E25" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="26" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E26" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="27" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E27" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="28" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E28" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="29" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E29" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="30" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E30" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="31" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E31" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="32" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E32" t="s">
+        <v>366</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="A4" r:id="rId1" xr:uid="{D1C23285-CAB8-401A-ABE0-736E097236DD}"/>
+    <hyperlink ref="A5" r:id="rId2" xr:uid="{41B8F711-48E4-4FD2-8267-082D73CFB4E7}"/>
+    <hyperlink ref="A3" r:id="rId3" xr:uid="{6C9F5C4F-8970-494B-8E6C-E89CB5678DDF}"/>
+    <hyperlink ref="A2" r:id="rId4" xr:uid="{87FA9602-2ECE-4ADD-BA31-DDC3DD127099}"/>
+    <hyperlink ref="A6" r:id="rId5" xr:uid="{CB9D2328-25FE-4EA7-8382-437A12AE6192}"/>
+    <hyperlink ref="A7" r:id="rId6" xr:uid="{4CE7CD25-59E8-43F6-A14E-8CEFEA87FE9B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -9622,11 +9852,20 @@
       <c r="C163" s="4" t="s">
         <v>580</v>
       </c>
+      <c r="D163" s="4">
+        <v>4</v>
+      </c>
       <c r="E163" s="4" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F163" s="4" t="s">
+        <v>593</v>
+      </c>
+      <c r="G163" s="5" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="4">
         <v>212</v>
       </c>
@@ -9636,8 +9875,17 @@
       <c r="C164" s="4" t="s">
         <v>580</v>
       </c>
+      <c r="D164" s="4">
+        <v>4</v>
+      </c>
       <c r="E164" s="4" t="s">
         <v>366</v>
+      </c>
+      <c r="F164" s="4" t="s">
+        <v>598</v>
+      </c>
+      <c r="G164" s="5" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
aoc and graph challenges
</commit_message>
<xml_diff>
--- a/docs/Programming Puzzles.xlsx
+++ b/docs/Programming Puzzles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\ProjectDSA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2372690-C255-4A30-9D9E-07ECAB16969A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{047EEC32-54C0-4C0E-8A6D-02F65329CEBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1686" uniqueCount="600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1730" uniqueCount="617">
   <si>
     <t>PLATFORM</t>
   </si>
@@ -1839,6 +1839,57 @@
   </si>
   <si>
     <t>Beautiful Code!</t>
+  </si>
+  <si>
+    <t>It's starting to make sense!</t>
+  </si>
+  <si>
+    <t>28/10/2026</t>
+  </si>
+  <si>
+    <t>Knight Attack</t>
+  </si>
+  <si>
+    <t>Can Color</t>
+  </si>
+  <si>
+    <t>Tolerant Teams</t>
+  </si>
+  <si>
+    <t>Rare Routing</t>
+  </si>
+  <si>
+    <t>Topological Order</t>
+  </si>
+  <si>
+    <t>Safe Cracking</t>
+  </si>
+  <si>
+    <t>String Search</t>
+  </si>
+  <si>
+    <t>Union Find Code I</t>
+  </si>
+  <si>
+    <t>Union Find Code II</t>
+  </si>
+  <si>
+    <t>Province Sizes</t>
+  </si>
+  <si>
+    <t>Extra Cable</t>
+  </si>
+  <si>
+    <t>Lowest Toll</t>
+  </si>
+  <si>
+    <t>Weighted Graph Min Path</t>
+  </si>
+  <si>
+    <t>Prefix Product</t>
+  </si>
+  <si>
+    <t>Shortest path, therefore we should use BFS.</t>
   </si>
 </sst>
 </file>
@@ -7167,7 +7218,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63392036-0DF4-41BC-932A-0EBA4F02E5CB}">
-  <dimension ref="A1:G202"/>
+  <dimension ref="A1:G197"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -9898,190 +9949,303 @@
       <c r="C165" s="4" t="s">
         <v>580</v>
       </c>
+      <c r="D165" s="4">
+        <v>3</v>
+      </c>
       <c r="E165" s="4" t="s">
         <v>366</v>
+      </c>
+      <c r="F165" s="4" t="s">
+        <v>598</v>
+      </c>
+      <c r="G165" s="5" t="s">
+        <v>600</v>
       </c>
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A166" s="4">
-        <v>214</v>
+        <v>215</v>
+      </c>
+      <c r="B166" s="4" t="s">
+        <v>602</v>
+      </c>
+      <c r="C166" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="D166" s="4">
+        <v>2</v>
+      </c>
+      <c r="E166" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="F166" s="4" t="s">
+        <v>601</v>
+      </c>
+      <c r="G166" s="5" t="s">
+        <v>616</v>
       </c>
     </row>
     <row r="167" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A167" s="4">
-        <v>215</v>
+        <v>216</v>
+      </c>
+      <c r="B167" s="4" t="s">
+        <v>603</v>
+      </c>
+      <c r="C167" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E167" s="4" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A168" s="4">
-        <v>216</v>
+        <v>217</v>
+      </c>
+      <c r="B168" s="4" t="s">
+        <v>604</v>
+      </c>
+      <c r="C168" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E168" s="4" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A169" s="4">
-        <v>217</v>
+        <v>218</v>
+      </c>
+      <c r="B169" s="4" t="s">
+        <v>605</v>
+      </c>
+      <c r="C169" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E169" s="4" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A170" s="4">
-        <v>218</v>
+        <v>219</v>
+      </c>
+      <c r="B170" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="C170" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E170" s="4" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A171" s="4">
-        <v>219</v>
+        <v>220</v>
+      </c>
+      <c r="B171" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="C171" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E171" s="4" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A172" s="4">
-        <v>220</v>
+        <v>221</v>
+      </c>
+      <c r="B172" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="C172" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E172" s="4" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A173" s="4">
-        <v>221</v>
+        <v>223</v>
+      </c>
+      <c r="B173" s="4" t="s">
+        <v>609</v>
+      </c>
+      <c r="C173" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E173" s="4" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="174" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A174" s="4">
-        <v>222</v>
+        <v>224</v>
+      </c>
+      <c r="B174" s="4" t="s">
+        <v>610</v>
+      </c>
+      <c r="C174" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E174" s="4" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A175" s="4">
-        <v>223</v>
+        <v>225</v>
+      </c>
+      <c r="B175" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="C175" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E175" s="4" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="176" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A176" s="4">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
+        <v>226</v>
+      </c>
+      <c r="B176" s="4" t="s">
+        <v>612</v>
+      </c>
+      <c r="C176" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E176" s="4" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="4">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
+        <v>228</v>
+      </c>
+      <c r="B177" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="C177" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E177" s="4" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="4">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+      <c r="B178" s="4" t="s">
+        <v>613</v>
+      </c>
+      <c r="C178" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E178" s="4" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="4">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
+        <v>232</v>
+      </c>
+      <c r="B179" s="4" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="4">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="4">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="4">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="4">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="4">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="4">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="4">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="4">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="4">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="4">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="4">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="4">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="4">
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="193" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A193" s="4">
-        <v>241</v>
+        <v>246</v>
       </c>
     </row>
     <row r="194" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A194" s="4">
-        <v>242</v>
+        <v>247</v>
       </c>
     </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A195" s="4">
-        <v>243</v>
+        <v>248</v>
       </c>
     </row>
     <row r="196" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A196" s="4">
-        <v>244</v>
-      </c>
+      <c r="A196" s="4"/>
     </row>
     <row r="197" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A197" s="4">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A198" s="4">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A199" s="4">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A200" s="4">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A201" s="4"/>
-    </row>
-    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A202" s="4"/>
+      <c r="A197" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
aoc and structy puzzles
</commit_message>
<xml_diff>
--- a/docs/Programming Puzzles.xlsx
+++ b/docs/Programming Puzzles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Projects\ProjectDSA\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{047EEC32-54C0-4C0E-8A6D-02F65329CEBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2418ACEE-408D-4EAD-BE00-9F8C206B20D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B7950DC0-5F1E-48EF-9340-8CAB6CE423A3}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1730" uniqueCount="617">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2199" uniqueCount="621">
   <si>
     <t>PLATFORM</t>
   </si>
@@ -1890,6 +1890,18 @@
   </si>
   <si>
     <t>Shortest path, therefore we should use BFS.</t>
+  </si>
+  <si>
+    <t>29/10/2026</t>
+  </si>
+  <si>
+    <t>DFS problem. Bipartite Graph.</t>
+  </si>
+  <si>
+    <t>30/10/2026</t>
+  </si>
+  <si>
+    <t>Bipartite Graph. Variation of the previous one.</t>
   </si>
 </sst>
 </file>
@@ -9995,8 +10007,17 @@
       <c r="C167" s="4" t="s">
         <v>431</v>
       </c>
+      <c r="D167" s="4">
+        <v>2</v>
+      </c>
       <c r="E167" s="4" t="s">
         <v>366</v>
+      </c>
+      <c r="F167" s="4" t="s">
+        <v>617</v>
+      </c>
+      <c r="G167" s="5" t="s">
+        <v>618</v>
       </c>
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.25">
@@ -10009,8 +10030,17 @@
       <c r="C168" s="4" t="s">
         <v>431</v>
       </c>
+      <c r="D168" s="4">
+        <v>2</v>
+      </c>
       <c r="E168" s="4" t="s">
         <v>366</v>
+      </c>
+      <c r="F168" s="4" t="s">
+        <v>619</v>
+      </c>
+      <c r="G168" s="5" t="s">
+        <v>620</v>
       </c>
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>